<commit_message>
B1: cardápio com consumo por pessoa e cesta completa; couvert não encontrado não entra como 0
A auditoria das planilhas agregadas achou 25 das 33 cestas somando couvert 0
quando o couvert não foi encontrado, contra a regra de 16/10 e contra a nota da
própria planilha. Escolha do autor: duas medidas. Consumo = bebida + entrada ou
prato (33 casas, mediana R$ 48,80); cesta completa = consumo + couvert
encontrado (8 casas, mediana R$ 74,25). Estatística descritiva e planilha
agregada do B1 refeitas; o site mantém a cesta casa a casa antiga até trocar o
rótulo. Divergências da auditoria registradas e listadas nas pendências.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RccbNmyt945Bi1GY3W8HKp
</commit_message>
<xml_diff>
--- a/dados/Dados agregados/B1_dados_agregados_completo.xlsx
+++ b/dados/Dados agregados/B1_dados_agregados_completo.xlsx
@@ -467,7 +467,7 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>11</col>
+      <col>13</col>
       <colOff>0</colOff>
       <row>1</row>
       <rowOff>0</rowOff>
@@ -500,12 +500,12 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>12</col>
+      <col>14</col>
       <colOff>0</colOff>
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5905500" cy="3273470"/>
+    <ext cx="5905500" cy="3263218"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -571,7 +571,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5905500" cy="2846112"/>
+    <ext cx="5905500" cy="3295926"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -3739,7 +3739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO58"/>
+  <dimension ref="A1:AR58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3783,6 +3783,9 @@
     <col width="13" customWidth="1" min="39" max="39"/>
     <col width="13" customWidth="1" min="40" max="40"/>
     <col width="13" customWidth="1" min="41" max="41"/>
+    <col width="13" customWidth="1" min="42" max="42"/>
+    <col width="13" customWidth="1" min="43" max="43"/>
+    <col width="13" customWidth="1" min="44" max="44"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3955,45 +3958,60 @@
       </c>
       <c r="AG2" s="2" t="inlineStr">
         <is>
-          <t>cesta baixa (R$)</t>
+          <t>consumo baixo (R$)</t>
         </is>
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>cesta mediana (R$)</t>
+          <t>consumo mediano (R$)</t>
         </is>
       </c>
       <c r="AI2" s="2" t="inlineStr">
         <is>
-          <t>cesta alta (R$)</t>
+          <t>consumo alto (R$)</t>
         </is>
       </c>
       <c r="AJ2" s="2" t="inlineStr">
         <is>
+          <t>cesta completa baixa (R$)</t>
+        </is>
+      </c>
+      <c r="AK2" s="2" t="inlineStr">
+        <is>
+          <t>cesta completa mediana (R$)</t>
+        </is>
+      </c>
+      <c r="AL2" s="2" t="inlineStr">
+        <is>
+          <t>cesta completa alta (R$)</t>
+        </is>
+      </c>
+      <c r="AM2" s="2" t="inlineStr">
+        <is>
           <t>hambúrguer (R$)</t>
         </is>
       </c>
-      <c r="AK2" s="2" t="inlineStr">
+      <c r="AN2" s="2" t="inlineStr">
         <is>
           <t>batata (R$)</t>
         </is>
       </c>
-      <c r="AL2" s="2" t="inlineStr">
+      <c r="AO2" s="2" t="inlineStr">
         <is>
           <t>cerveja (R$)</t>
         </is>
       </c>
-      <c r="AM2" s="2" t="inlineStr">
+      <c r="AP2" s="2" t="inlineStr">
         <is>
           <t>refrigerante (R$)</t>
         </is>
       </c>
-      <c r="AN2" s="2" t="inlineStr">
+      <c r="AQ2" s="2" t="inlineStr">
         <is>
           <t>drinks (R$)</t>
         </is>
       </c>
-      <c r="AO2" s="2" t="inlineStr">
+      <c r="AR2" s="2" t="inlineStr">
         <is>
           <t>títulos no acervo</t>
         </is>
@@ -4109,20 +4127,23 @@
       <c r="AI3" s="14" t="n">
         <v>45</v>
       </c>
-      <c r="AJ3" s="14" t="n">
+      <c r="AJ3" s="14" t="n"/>
+      <c r="AK3" s="14" t="n"/>
+      <c r="AL3" s="14" t="n"/>
+      <c r="AM3" s="14" t="n">
         <v>32</v>
       </c>
-      <c r="AK3" s="14" t="n">
+      <c r="AN3" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="AL3" s="14" t="n">
+      <c r="AO3" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="AM3" s="14" t="n">
+      <c r="AP3" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="AN3" s="14" t="n"/>
-      <c r="AO3" s="15" t="n"/>
+      <c r="AQ3" s="14" t="n"/>
+      <c r="AR3" s="15" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
@@ -4225,7 +4246,10 @@
       <c r="AL4" s="14" t="n"/>
       <c r="AM4" s="14" t="n"/>
       <c r="AN4" s="14" t="n"/>
-      <c r="AO4" s="15" t="n"/>
+      <c r="AO4" s="14" t="n"/>
+      <c r="AP4" s="14" t="n"/>
+      <c r="AQ4" s="14" t="n"/>
+      <c r="AR4" s="15" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
@@ -4339,14 +4363,17 @@
       </c>
       <c r="AJ5" s="14" t="n"/>
       <c r="AK5" s="14" t="n"/>
-      <c r="AL5" s="14" t="n">
+      <c r="AL5" s="14" t="n"/>
+      <c r="AM5" s="14" t="n"/>
+      <c r="AN5" s="14" t="n"/>
+      <c r="AO5" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="AM5" s="14" t="n">
+      <c r="AP5" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="AN5" s="14" t="n"/>
-      <c r="AO5" s="15" t="n"/>
+      <c r="AQ5" s="14" t="n"/>
+      <c r="AR5" s="15" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
@@ -4452,30 +4479,39 @@
         <v>33</v>
       </c>
       <c r="AG6" s="14" t="n">
+        <v>40.75</v>
+      </c>
+      <c r="AH6" s="14" t="n">
+        <v>50</v>
+      </c>
+      <c r="AI6" s="14" t="n">
+        <v>60.25</v>
+      </c>
+      <c r="AJ6" s="14" t="n">
         <v>54.5</v>
       </c>
-      <c r="AH6" s="14" t="n">
+      <c r="AK6" s="14" t="n">
         <v>67.5</v>
       </c>
-      <c r="AI6" s="14" t="n">
+      <c r="AL6" s="14" t="n">
         <v>81.5</v>
       </c>
-      <c r="AJ6" s="14" t="n">
+      <c r="AM6" s="14" t="n">
         <v>45</v>
       </c>
-      <c r="AK6" s="14" t="n">
+      <c r="AN6" s="14" t="n">
         <v>30.5</v>
       </c>
-      <c r="AL6" s="14" t="n">
+      <c r="AO6" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="AM6" s="14" t="n">
+      <c r="AP6" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="AN6" s="14" t="n">
+      <c r="AQ6" s="14" t="n">
         <v>22</v>
       </c>
-      <c r="AO6" s="15" t="n">
+      <c r="AR6" s="15" t="n">
         <v>150</v>
       </c>
     </row>
@@ -4583,26 +4619,35 @@
         <v>31</v>
       </c>
       <c r="AG7" s="14" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="AH7" s="14" t="n">
+        <v>40</v>
+      </c>
+      <c r="AI7" s="14" t="n">
+        <v>46.75</v>
+      </c>
+      <c r="AJ7" s="14" t="n">
         <v>64.5</v>
       </c>
-      <c r="AH7" s="14" t="n">
+      <c r="AK7" s="14" t="n">
         <v>70</v>
       </c>
-      <c r="AI7" s="14" t="n">
+      <c r="AL7" s="14" t="n">
         <v>76.75</v>
       </c>
-      <c r="AJ7" s="14" t="n"/>
-      <c r="AK7" s="14" t="n"/>
-      <c r="AL7" s="14" t="n">
+      <c r="AM7" s="14" t="n"/>
+      <c r="AN7" s="14" t="n"/>
+      <c r="AO7" s="14" t="n">
         <v>8.5</v>
       </c>
-      <c r="AM7" s="14" t="n">
+      <c r="AP7" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="AN7" s="14" t="n">
+      <c r="AQ7" s="14" t="n">
         <v>14</v>
       </c>
-      <c r="AO7" s="15" t="n">
+      <c r="AR7" s="15" t="n">
         <v>952</v>
       </c>
     </row>
@@ -4717,17 +4762,20 @@
         <v>84.5</v>
       </c>
       <c r="AJ8" s="14" t="n"/>
-      <c r="AK8" s="14" t="n">
+      <c r="AK8" s="14" t="n"/>
+      <c r="AL8" s="14" t="n"/>
+      <c r="AM8" s="14" t="n"/>
+      <c r="AN8" s="14" t="n">
         <v>25.5</v>
       </c>
-      <c r="AL8" s="14" t="n">
+      <c r="AO8" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="AM8" s="14" t="n">
+      <c r="AP8" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="AN8" s="14" t="n"/>
-      <c r="AO8" s="15" t="n"/>
+      <c r="AQ8" s="14" t="n"/>
+      <c r="AR8" s="15" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="13" t="inlineStr">
@@ -4828,7 +4876,10 @@
       <c r="AL9" s="14" t="n"/>
       <c r="AM9" s="14" t="n"/>
       <c r="AN9" s="14" t="n"/>
-      <c r="AO9" s="15" t="n">
+      <c r="AO9" s="14" t="n"/>
+      <c r="AP9" s="14" t="n"/>
+      <c r="AQ9" s="14" t="n"/>
+      <c r="AR9" s="15" t="n">
         <v>214</v>
       </c>
     </row>
@@ -4942,22 +4993,25 @@
       <c r="AI10" s="14" t="n">
         <v>45</v>
       </c>
-      <c r="AJ10" s="14" t="n">
+      <c r="AJ10" s="14" t="n"/>
+      <c r="AK10" s="14" t="n"/>
+      <c r="AL10" s="14" t="n"/>
+      <c r="AM10" s="14" t="n">
         <v>29.5</v>
       </c>
-      <c r="AK10" s="14" t="n">
+      <c r="AN10" s="14" t="n">
         <v>26.5</v>
       </c>
-      <c r="AL10" s="14" t="n">
+      <c r="AO10" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="AM10" s="14" t="n">
+      <c r="AP10" s="14" t="n">
         <v>7.5</v>
       </c>
-      <c r="AN10" s="14" t="n">
+      <c r="AQ10" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="AO10" s="15" t="n">
+      <c r="AR10" s="15" t="n">
         <v>1833</v>
       </c>
     </row>
@@ -5050,7 +5104,10 @@
       <c r="AL11" s="14" t="n"/>
       <c r="AM11" s="14" t="n"/>
       <c r="AN11" s="14" t="n"/>
-      <c r="AO11" s="15" t="n"/>
+      <c r="AO11" s="14" t="n"/>
+      <c r="AP11" s="14" t="n"/>
+      <c r="AQ11" s="14" t="n"/>
+      <c r="AR11" s="15" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
@@ -5162,18 +5219,21 @@
       <c r="AI12" s="14" t="n">
         <v>37.5</v>
       </c>
-      <c r="AJ12" s="14" t="n">
+      <c r="AJ12" s="14" t="n"/>
+      <c r="AK12" s="14" t="n"/>
+      <c r="AL12" s="14" t="n"/>
+      <c r="AM12" s="14" t="n">
         <v>34</v>
       </c>
-      <c r="AK12" s="14" t="n">
+      <c r="AN12" s="14" t="n">
         <v>19</v>
       </c>
-      <c r="AL12" s="14" t="n">
+      <c r="AO12" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="AM12" s="14" t="n"/>
-      <c r="AN12" s="14" t="n"/>
-      <c r="AO12" s="15" t="n">
+      <c r="AP12" s="14" t="n"/>
+      <c r="AQ12" s="14" t="n"/>
+      <c r="AR12" s="15" t="n">
         <v>312</v>
       </c>
     </row>
@@ -5287,22 +5347,25 @@
       <c r="AI13" s="14" t="n">
         <v>60.5</v>
       </c>
-      <c r="AJ13" s="14" t="n">
+      <c r="AJ13" s="14" t="n"/>
+      <c r="AK13" s="14" t="n"/>
+      <c r="AL13" s="14" t="n"/>
+      <c r="AM13" s="14" t="n">
         <v>45</v>
       </c>
-      <c r="AK13" s="14" t="n">
+      <c r="AN13" s="14" t="n">
         <v>35</v>
       </c>
-      <c r="AL13" s="14" t="n">
+      <c r="AO13" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="AM13" s="14" t="n">
+      <c r="AP13" s="14" t="n">
         <v>8.9</v>
       </c>
-      <c r="AN13" s="14" t="n">
+      <c r="AQ13" s="14" t="n">
         <v>28</v>
       </c>
-      <c r="AO13" s="15" t="n">
+      <c r="AR13" s="15" t="n">
         <v>370</v>
       </c>
     </row>
@@ -5408,30 +5471,39 @@
         <v>35</v>
       </c>
       <c r="AG14" s="14" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="AH14" s="14" t="n">
+        <v>48</v>
+      </c>
+      <c r="AI14" s="14" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="AJ14" s="14" t="n">
         <v>56.75</v>
       </c>
-      <c r="AH14" s="14" t="n">
+      <c r="AK14" s="14" t="n">
         <v>73.5</v>
       </c>
-      <c r="AI14" s="14" t="n">
+      <c r="AL14" s="14" t="n">
         <v>81.25</v>
       </c>
-      <c r="AJ14" s="14" t="n">
+      <c r="AM14" s="14" t="n">
         <v>40</v>
       </c>
-      <c r="AK14" s="14" t="n">
+      <c r="AN14" s="14" t="n">
         <v>31</v>
       </c>
-      <c r="AL14" s="14" t="n">
+      <c r="AO14" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="AM14" s="14" t="n">
+      <c r="AP14" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="AN14" s="14" t="n">
+      <c r="AQ14" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="AO14" s="15" t="n">
+      <c r="AR14" s="15" t="n">
         <v>468</v>
       </c>
     </row>
@@ -5541,20 +5613,23 @@
       <c r="AI15" s="14" t="n">
         <v>71.5</v>
       </c>
-      <c r="AJ15" s="14" t="n">
+      <c r="AJ15" s="14" t="n"/>
+      <c r="AK15" s="14" t="n"/>
+      <c r="AL15" s="14" t="n"/>
+      <c r="AM15" s="14" t="n">
         <v>42</v>
       </c>
-      <c r="AK15" s="14" t="n"/>
-      <c r="AL15" s="14" t="n">
+      <c r="AN15" s="14" t="n"/>
+      <c r="AO15" s="14" t="n">
         <v>12.5</v>
       </c>
-      <c r="AM15" s="14" t="n">
+      <c r="AP15" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="AN15" s="14" t="n">
+      <c r="AQ15" s="14" t="n">
         <v>26</v>
       </c>
-      <c r="AO15" s="15" t="n">
+      <c r="AR15" s="15" t="n">
         <v>588</v>
       </c>
     </row>
@@ -5662,26 +5737,35 @@
         <v>50</v>
       </c>
       <c r="AG16" s="14" t="n">
+        <v>54.75</v>
+      </c>
+      <c r="AH16" s="14" t="n">
+        <v>68</v>
+      </c>
+      <c r="AI16" s="14" t="n">
+        <v>80</v>
+      </c>
+      <c r="AJ16" s="14" t="n">
         <v>71</v>
       </c>
-      <c r="AH16" s="14" t="n">
+      <c r="AK16" s="14" t="n">
         <v>85.5</v>
       </c>
-      <c r="AI16" s="14" t="n">
+      <c r="AL16" s="14" t="n">
         <v>98.75</v>
       </c>
-      <c r="AJ16" s="14" t="n">
+      <c r="AM16" s="14" t="n">
         <v>50</v>
       </c>
-      <c r="AK16" s="14" t="n"/>
-      <c r="AL16" s="14" t="n">
+      <c r="AN16" s="14" t="n"/>
+      <c r="AO16" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="AM16" s="14" t="n"/>
-      <c r="AN16" s="14" t="n">
+      <c r="AP16" s="14" t="n"/>
+      <c r="AQ16" s="14" t="n">
         <v>25</v>
       </c>
-      <c r="AO16" s="15" t="n">
+      <c r="AR16" s="15" t="n">
         <v>190</v>
       </c>
     </row>
@@ -5786,7 +5870,10 @@
       <c r="AL17" s="14" t="n"/>
       <c r="AM17" s="14" t="n"/>
       <c r="AN17" s="14" t="n"/>
-      <c r="AO17" s="15" t="n"/>
+      <c r="AO17" s="14" t="n"/>
+      <c r="AP17" s="14" t="n"/>
+      <c r="AQ17" s="14" t="n"/>
+      <c r="AR17" s="15" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
@@ -5886,30 +5973,39 @@
         <v>35</v>
       </c>
       <c r="AG18" s="14" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="AH18" s="14" t="n">
+        <v>55</v>
+      </c>
+      <c r="AI18" s="14" t="n">
+        <v>67.5</v>
+      </c>
+      <c r="AJ18" s="14" t="n">
         <v>58.5</v>
       </c>
-      <c r="AH18" s="14" t="n">
+      <c r="AK18" s="14" t="n">
         <v>75</v>
       </c>
-      <c r="AI18" s="14" t="n">
+      <c r="AL18" s="14" t="n">
         <v>87.5</v>
       </c>
-      <c r="AJ18" s="14" t="n">
+      <c r="AM18" s="14" t="n">
         <v>42</v>
       </c>
-      <c r="AK18" s="14" t="n">
+      <c r="AN18" s="14" t="n">
         <v>37.5</v>
       </c>
-      <c r="AL18" s="14" t="n">
+      <c r="AO18" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="AM18" s="14" t="n">
+      <c r="AP18" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="AN18" s="14" t="n">
+      <c r="AQ18" s="14" t="n">
         <v>25</v>
       </c>
-      <c r="AO18" s="15" t="n">
+      <c r="AR18" s="15" t="n">
         <v>192</v>
       </c>
     </row>
@@ -6002,7 +6098,10 @@
       <c r="AL19" s="14" t="n"/>
       <c r="AM19" s="14" t="n"/>
       <c r="AN19" s="14" t="n"/>
-      <c r="AO19" s="15" t="n">
+      <c r="AO19" s="14" t="n"/>
+      <c r="AP19" s="14" t="n"/>
+      <c r="AQ19" s="14" t="n"/>
+      <c r="AR19" s="15" t="n">
         <v>362</v>
       </c>
     </row>
@@ -6110,30 +6209,39 @@
         <v>52</v>
       </c>
       <c r="AG20" s="14" t="n">
+        <v>56.5</v>
+      </c>
+      <c r="AH20" s="14" t="n">
+        <v>77</v>
+      </c>
+      <c r="AI20" s="14" t="n">
+        <v>96</v>
+      </c>
+      <c r="AJ20" s="14" t="n">
         <v>74</v>
       </c>
-      <c r="AH20" s="14" t="n">
+      <c r="AK20" s="14" t="n">
         <v>97</v>
       </c>
-      <c r="AI20" s="14" t="n">
+      <c r="AL20" s="14" t="n">
         <v>121</v>
       </c>
-      <c r="AJ20" s="14" t="n">
+      <c r="AM20" s="14" t="n">
         <v>54</v>
       </c>
-      <c r="AK20" s="14" t="n">
+      <c r="AN20" s="14" t="n">
         <v>40</v>
       </c>
-      <c r="AL20" s="14" t="n">
+      <c r="AO20" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="AM20" s="14" t="n">
+      <c r="AP20" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="AN20" s="14" t="n">
+      <c r="AQ20" s="14" t="n">
         <v>28</v>
       </c>
-      <c r="AO20" s="15" t="n">
+      <c r="AR20" s="15" t="n">
         <v>836</v>
       </c>
     </row>
@@ -6238,7 +6346,10 @@
       <c r="AL21" s="14" t="n"/>
       <c r="AM21" s="14" t="n"/>
       <c r="AN21" s="14" t="n"/>
-      <c r="AO21" s="15" t="n"/>
+      <c r="AO21" s="14" t="n"/>
+      <c r="AP21" s="14" t="n"/>
+      <c r="AQ21" s="14" t="n"/>
+      <c r="AR21" s="15" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
@@ -6350,20 +6461,23 @@
       <c r="AI22" s="14" t="n">
         <v>54.5</v>
       </c>
-      <c r="AJ22" s="14" t="n">
+      <c r="AJ22" s="14" t="n"/>
+      <c r="AK22" s="14" t="n"/>
+      <c r="AL22" s="14" t="n"/>
+      <c r="AM22" s="14" t="n">
         <v>38</v>
       </c>
-      <c r="AK22" s="14" t="n">
+      <c r="AN22" s="14" t="n">
         <v>24</v>
       </c>
-      <c r="AL22" s="14" t="n">
+      <c r="AO22" s="14" t="n">
         <v>16.5</v>
       </c>
-      <c r="AM22" s="14" t="n">
+      <c r="AP22" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="AN22" s="14" t="n"/>
-      <c r="AO22" s="15" t="n">
+      <c r="AQ22" s="14" t="n"/>
+      <c r="AR22" s="15" t="n">
         <v>780</v>
       </c>
     </row>
@@ -6468,7 +6582,10 @@
       <c r="AL23" s="14" t="n"/>
       <c r="AM23" s="14" t="n"/>
       <c r="AN23" s="14" t="n"/>
-      <c r="AO23" s="15" t="n"/>
+      <c r="AO23" s="14" t="n"/>
+      <c r="AP23" s="14" t="n"/>
+      <c r="AQ23" s="14" t="n"/>
+      <c r="AR23" s="15" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="13" t="inlineStr">
@@ -6571,7 +6688,10 @@
       <c r="AL24" s="14" t="n"/>
       <c r="AM24" s="14" t="n"/>
       <c r="AN24" s="14" t="n"/>
-      <c r="AO24" s="15" t="n"/>
+      <c r="AO24" s="14" t="n"/>
+      <c r="AP24" s="14" t="n"/>
+      <c r="AQ24" s="14" t="n"/>
+      <c r="AR24" s="15" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="13" t="inlineStr">
@@ -6668,7 +6788,10 @@
       <c r="AL25" s="14" t="n"/>
       <c r="AM25" s="14" t="n"/>
       <c r="AN25" s="14" t="n"/>
-      <c r="AO25" s="15" t="n">
+      <c r="AO25" s="14" t="n"/>
+      <c r="AP25" s="14" t="n"/>
+      <c r="AQ25" s="14" t="n"/>
+      <c r="AR25" s="15" t="n">
         <v>1357</v>
       </c>
     </row>
@@ -6776,30 +6899,39 @@
         <v>45</v>
       </c>
       <c r="AG26" s="14" t="n">
+        <v>46</v>
+      </c>
+      <c r="AH26" s="14" t="n">
+        <v>56</v>
+      </c>
+      <c r="AI26" s="14" t="n">
+        <v>78</v>
+      </c>
+      <c r="AJ26" s="14" t="n">
         <v>52.25</v>
       </c>
-      <c r="AH26" s="14" t="n">
+      <c r="AK26" s="14" t="n">
         <v>68.5</v>
       </c>
-      <c r="AI26" s="14" t="n">
+      <c r="AL26" s="14" t="n">
         <v>96.75</v>
       </c>
-      <c r="AJ26" s="14" t="n">
+      <c r="AM26" s="14" t="n">
         <v>52.5</v>
       </c>
-      <c r="AK26" s="14" t="n">
+      <c r="AN26" s="14" t="n">
         <v>28.5</v>
       </c>
-      <c r="AL26" s="14" t="n">
+      <c r="AO26" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="AM26" s="14" t="n">
+      <c r="AP26" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="AN26" s="14" t="n">
+      <c r="AQ26" s="14" t="n">
         <v>25</v>
       </c>
-      <c r="AO26" s="15" t="n">
+      <c r="AR26" s="15" t="n">
         <v>540</v>
       </c>
     </row>
@@ -6913,22 +7045,25 @@
       <c r="AI27" s="14" t="n">
         <v>76</v>
       </c>
-      <c r="AJ27" s="14" t="n">
+      <c r="AJ27" s="14" t="n"/>
+      <c r="AK27" s="14" t="n"/>
+      <c r="AL27" s="14" t="n"/>
+      <c r="AM27" s="14" t="n">
         <v>49.5</v>
       </c>
-      <c r="AK27" s="14" t="n">
+      <c r="AN27" s="14" t="n">
         <v>39</v>
       </c>
-      <c r="AL27" s="14" t="n">
+      <c r="AO27" s="14" t="n">
         <v>16</v>
       </c>
-      <c r="AM27" s="14" t="n">
+      <c r="AP27" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="AN27" s="14" t="n">
+      <c r="AQ27" s="14" t="n">
         <v>36.5</v>
       </c>
-      <c r="AO27" s="15" t="n">
+      <c r="AR27" s="15" t="n">
         <v>934</v>
       </c>
     </row>
@@ -7031,7 +7166,10 @@
       <c r="AL28" s="14" t="n"/>
       <c r="AM28" s="14" t="n"/>
       <c r="AN28" s="14" t="n"/>
-      <c r="AO28" s="15" t="n"/>
+      <c r="AO28" s="14" t="n"/>
+      <c r="AP28" s="14" t="n"/>
+      <c r="AQ28" s="14" t="n"/>
+      <c r="AR28" s="15" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="13" t="inlineStr">
@@ -7144,15 +7282,18 @@
         <v>78</v>
       </c>
       <c r="AJ29" s="14" t="n"/>
-      <c r="AK29" s="14" t="n">
-        <v>68</v>
-      </c>
+      <c r="AK29" s="14" t="n"/>
       <c r="AL29" s="14" t="n"/>
       <c r="AM29" s="14" t="n"/>
       <c r="AN29" s="14" t="n">
+        <v>68</v>
+      </c>
+      <c r="AO29" s="14" t="n"/>
+      <c r="AP29" s="14" t="n"/>
+      <c r="AQ29" s="14" t="n">
         <v>36</v>
       </c>
-      <c r="AO29" s="15" t="n"/>
+      <c r="AR29" s="15" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
@@ -7264,22 +7405,25 @@
       <c r="AI30" s="14" t="n">
         <v>83.55</v>
       </c>
-      <c r="AJ30" s="14" t="n">
+      <c r="AJ30" s="14" t="n"/>
+      <c r="AK30" s="14" t="n"/>
+      <c r="AL30" s="14" t="n"/>
+      <c r="AM30" s="14" t="n">
         <v>43.9</v>
       </c>
-      <c r="AK30" s="14" t="n">
+      <c r="AN30" s="14" t="n">
         <v>39.9</v>
       </c>
-      <c r="AL30" s="14" t="n">
+      <c r="AO30" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="AM30" s="14" t="n">
+      <c r="AP30" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="AN30" s="14" t="n">
+      <c r="AQ30" s="14" t="n">
         <v>37.9</v>
       </c>
-      <c r="AO30" s="15" t="n">
+      <c r="AR30" s="15" t="n">
         <v>225</v>
       </c>
     </row>
@@ -7393,22 +7537,25 @@
       <c r="AI31" s="14" t="n">
         <v>69</v>
       </c>
-      <c r="AJ31" s="14" t="n">
+      <c r="AJ31" s="14" t="n"/>
+      <c r="AK31" s="14" t="n"/>
+      <c r="AL31" s="14" t="n"/>
+      <c r="AM31" s="14" t="n">
         <v>28</v>
       </c>
-      <c r="AK31" s="14" t="n">
+      <c r="AN31" s="14" t="n">
         <v>33</v>
       </c>
-      <c r="AL31" s="14" t="n">
+      <c r="AO31" s="14" t="n">
         <v>22</v>
       </c>
-      <c r="AM31" s="14" t="n">
+      <c r="AP31" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="AN31" s="14" t="n">
+      <c r="AQ31" s="14" t="n">
         <v>30</v>
       </c>
-      <c r="AO31" s="15" t="n"/>
+      <c r="AR31" s="15" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="13" t="inlineStr">
@@ -7520,22 +7667,25 @@
       <c r="AI32" s="14" t="n">
         <v>60</v>
       </c>
-      <c r="AJ32" s="14" t="n">
+      <c r="AJ32" s="14" t="n"/>
+      <c r="AK32" s="14" t="n"/>
+      <c r="AL32" s="14" t="n"/>
+      <c r="AM32" s="14" t="n">
         <v>29</v>
       </c>
-      <c r="AK32" s="14" t="n">
+      <c r="AN32" s="14" t="n">
         <v>50</v>
       </c>
-      <c r="AL32" s="14" t="n">
+      <c r="AO32" s="14" t="n">
         <v>17</v>
       </c>
-      <c r="AM32" s="14" t="n">
+      <c r="AP32" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="AN32" s="14" t="n">
+      <c r="AQ32" s="14" t="n">
         <v>21.5</v>
       </c>
-      <c r="AO32" s="15" t="n">
+      <c r="AR32" s="15" t="n">
         <v>239</v>
       </c>
     </row>
@@ -7649,22 +7799,25 @@
       <c r="AI33" s="14" t="n">
         <v>52.5</v>
       </c>
-      <c r="AJ33" s="14" t="n">
+      <c r="AJ33" s="14" t="n"/>
+      <c r="AK33" s="14" t="n"/>
+      <c r="AL33" s="14" t="n"/>
+      <c r="AM33" s="14" t="n">
         <v>31</v>
       </c>
-      <c r="AK33" s="14" t="n">
+      <c r="AN33" s="14" t="n">
         <v>30</v>
       </c>
-      <c r="AL33" s="14" t="n">
+      <c r="AO33" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="AM33" s="14" t="n">
+      <c r="AP33" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="AN33" s="14" t="n">
+      <c r="AQ33" s="14" t="n">
         <v>28</v>
       </c>
-      <c r="AO33" s="15" t="n">
+      <c r="AR33" s="15" t="n">
         <v>90</v>
       </c>
     </row>
@@ -7778,16 +7931,19 @@
       <c r="AI34" s="14" t="n">
         <v>76.8</v>
       </c>
-      <c r="AJ34" s="14" t="n">
+      <c r="AJ34" s="14" t="n"/>
+      <c r="AK34" s="14" t="n"/>
+      <c r="AL34" s="14" t="n"/>
+      <c r="AM34" s="14" t="n">
         <v>38</v>
       </c>
-      <c r="AK34" s="14" t="n">
+      <c r="AN34" s="14" t="n">
         <v>24.9</v>
       </c>
-      <c r="AL34" s="14" t="n"/>
-      <c r="AM34" s="14" t="n"/>
-      <c r="AN34" s="14" t="n"/>
-      <c r="AO34" s="15" t="n"/>
+      <c r="AO34" s="14" t="n"/>
+      <c r="AP34" s="14" t="n"/>
+      <c r="AQ34" s="14" t="n"/>
+      <c r="AR34" s="15" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="13" t="inlineStr">
@@ -7890,7 +8046,10 @@
       <c r="AL35" s="14" t="n"/>
       <c r="AM35" s="14" t="n"/>
       <c r="AN35" s="14" t="n"/>
-      <c r="AO35" s="15" t="n"/>
+      <c r="AO35" s="14" t="n"/>
+      <c r="AP35" s="14" t="n"/>
+      <c r="AQ35" s="14" t="n"/>
+      <c r="AR35" s="15" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="13" t="inlineStr">
@@ -8002,20 +8161,23 @@
       <c r="AI36" s="14" t="n">
         <v>41.9</v>
       </c>
-      <c r="AJ36" s="14" t="n">
+      <c r="AJ36" s="14" t="n"/>
+      <c r="AK36" s="14" t="n"/>
+      <c r="AL36" s="14" t="n"/>
+      <c r="AM36" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="AK36" s="14" t="n">
+      <c r="AN36" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="AL36" s="14" t="n">
+      <c r="AO36" s="14" t="n">
         <v>6.5</v>
       </c>
-      <c r="AM36" s="14" t="n">
+      <c r="AP36" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="AN36" s="14" t="n"/>
-      <c r="AO36" s="15" t="n"/>
+      <c r="AQ36" s="14" t="n"/>
+      <c r="AR36" s="15" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="13" t="inlineStr">
@@ -8122,11 +8284,14 @@
       <c r="AJ37" s="14" t="n"/>
       <c r="AK37" s="14" t="n"/>
       <c r="AL37" s="14" t="n"/>
-      <c r="AM37" s="14" t="n">
+      <c r="AM37" s="14" t="n"/>
+      <c r="AN37" s="14" t="n"/>
+      <c r="AO37" s="14" t="n"/>
+      <c r="AP37" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="AN37" s="14" t="n"/>
-      <c r="AO37" s="15" t="n">
+      <c r="AQ37" s="14" t="n"/>
+      <c r="AR37" s="15" t="n">
         <v>331</v>
       </c>
     </row>
@@ -8241,21 +8406,30 @@
         <v>92.5</v>
       </c>
       <c r="AJ38" s="14" t="n">
+        <v>63</v>
+      </c>
+      <c r="AK38" s="14" t="n">
+        <v>82</v>
+      </c>
+      <c r="AL38" s="14" t="n">
+        <v>92.5</v>
+      </c>
+      <c r="AM38" s="14" t="n">
         <v>42</v>
       </c>
-      <c r="AK38" s="14" t="n">
+      <c r="AN38" s="14" t="n">
         <v>48</v>
       </c>
-      <c r="AL38" s="14" t="n">
+      <c r="AO38" s="14" t="n">
         <v>18.5</v>
       </c>
-      <c r="AM38" s="14" t="n">
+      <c r="AP38" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="AN38" s="14" t="n">
+      <c r="AQ38" s="14" t="n">
         <v>36</v>
       </c>
-      <c r="AO38" s="15" t="n">
+      <c r="AR38" s="15" t="n">
         <v>199</v>
       </c>
     </row>
@@ -8360,7 +8534,10 @@
       <c r="AL39" s="14" t="n"/>
       <c r="AM39" s="14" t="n"/>
       <c r="AN39" s="14" t="n"/>
-      <c r="AO39" s="15" t="n">
+      <c r="AO39" s="14" t="n"/>
+      <c r="AP39" s="14" t="n"/>
+      <c r="AQ39" s="14" t="n"/>
+      <c r="AR39" s="15" t="n">
         <v>59</v>
       </c>
     </row>
@@ -8465,7 +8642,10 @@
       <c r="AL40" s="14" t="n"/>
       <c r="AM40" s="14" t="n"/>
       <c r="AN40" s="14" t="n"/>
-      <c r="AO40" s="15" t="n">
+      <c r="AO40" s="14" t="n"/>
+      <c r="AP40" s="14" t="n"/>
+      <c r="AQ40" s="14" t="n"/>
+      <c r="AR40" s="15" t="n">
         <v>227</v>
       </c>
     </row>
@@ -8579,20 +8759,23 @@
       <c r="AI41" s="14" t="n">
         <v>53.5</v>
       </c>
-      <c r="AJ41" s="14" t="n">
+      <c r="AJ41" s="14" t="n"/>
+      <c r="AK41" s="14" t="n"/>
+      <c r="AL41" s="14" t="n"/>
+      <c r="AM41" s="14" t="n">
         <v>38.9</v>
       </c>
-      <c r="AK41" s="14" t="n">
+      <c r="AN41" s="14" t="n">
         <v>33</v>
       </c>
-      <c r="AL41" s="14" t="n">
+      <c r="AO41" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="AM41" s="14" t="n">
+      <c r="AP41" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="AN41" s="14" t="n"/>
-      <c r="AO41" s="15" t="n">
+      <c r="AQ41" s="14" t="n"/>
+      <c r="AR41" s="15" t="n">
         <v>633</v>
       </c>
     </row>
@@ -8707,17 +8890,20 @@
         <v>34.5</v>
       </c>
       <c r="AJ42" s="14" t="n"/>
-      <c r="AK42" s="14" t="n">
+      <c r="AK42" s="14" t="n"/>
+      <c r="AL42" s="14" t="n"/>
+      <c r="AM42" s="14" t="n"/>
+      <c r="AN42" s="14" t="n">
         <v>16</v>
       </c>
-      <c r="AL42" s="14" t="n">
+      <c r="AO42" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="AM42" s="14" t="n">
+      <c r="AP42" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="AN42" s="14" t="n"/>
-      <c r="AO42" s="15" t="n">
+      <c r="AQ42" s="14" t="n"/>
+      <c r="AR42" s="15" t="n">
         <v>438</v>
       </c>
     </row>
@@ -8819,16 +9005,19 @@
       <c r="AG43" s="14" t="n"/>
       <c r="AH43" s="14" t="n"/>
       <c r="AI43" s="14" t="n"/>
-      <c r="AJ43" s="14" t="n">
+      <c r="AJ43" s="14" t="n"/>
+      <c r="AK43" s="14" t="n"/>
+      <c r="AL43" s="14" t="n"/>
+      <c r="AM43" s="14" t="n">
         <v>48</v>
       </c>
-      <c r="AK43" s="14" t="n">
+      <c r="AN43" s="14" t="n">
         <v>35</v>
       </c>
-      <c r="AL43" s="14" t="n"/>
-      <c r="AM43" s="14" t="n"/>
-      <c r="AN43" s="14" t="n"/>
-      <c r="AO43" s="15" t="n">
+      <c r="AO43" s="14" t="n"/>
+      <c r="AP43" s="14" t="n"/>
+      <c r="AQ43" s="14" t="n"/>
+      <c r="AR43" s="15" t="n">
         <v>221</v>
       </c>
     </row>
@@ -8933,7 +9122,10 @@
       <c r="AL44" s="14" t="n"/>
       <c r="AM44" s="14" t="n"/>
       <c r="AN44" s="14" t="n"/>
-      <c r="AO44" s="15" t="n"/>
+      <c r="AO44" s="14" t="n"/>
+      <c r="AP44" s="14" t="n"/>
+      <c r="AQ44" s="14" t="n"/>
+      <c r="AR44" s="15" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="13" t="inlineStr">
@@ -9044,17 +9236,20 @@
         <v>30.25</v>
       </c>
       <c r="AJ45" s="14" t="n"/>
-      <c r="AK45" s="14" t="n">
+      <c r="AK45" s="14" t="n"/>
+      <c r="AL45" s="14" t="n"/>
+      <c r="AM45" s="14" t="n"/>
+      <c r="AN45" s="14" t="n">
         <v>18</v>
       </c>
-      <c r="AL45" s="14" t="n">
+      <c r="AO45" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="AM45" s="14" t="n">
+      <c r="AP45" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="AN45" s="14" t="n"/>
-      <c r="AO45" s="15" t="n"/>
+      <c r="AQ45" s="14" t="n"/>
+      <c r="AR45" s="15" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="13" t="inlineStr">
@@ -9167,11 +9362,14 @@
       <c r="AJ46" s="14" t="n"/>
       <c r="AK46" s="14" t="n"/>
       <c r="AL46" s="14" t="n"/>
-      <c r="AM46" s="14" t="n">
+      <c r="AM46" s="14" t="n"/>
+      <c r="AN46" s="14" t="n"/>
+      <c r="AO46" s="14" t="n"/>
+      <c r="AP46" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="AN46" s="14" t="n"/>
-      <c r="AO46" s="15" t="n">
+      <c r="AQ46" s="14" t="n"/>
+      <c r="AR46" s="15" t="n">
         <v>270</v>
       </c>
     </row>
@@ -9283,22 +9481,25 @@
       <c r="AI47" s="14" t="n">
         <v>58</v>
       </c>
-      <c r="AJ47" s="14" t="n">
+      <c r="AJ47" s="14" t="n"/>
+      <c r="AK47" s="14" t="n"/>
+      <c r="AL47" s="14" t="n"/>
+      <c r="AM47" s="14" t="n">
         <v>32</v>
       </c>
-      <c r="AK47" s="14" t="n">
+      <c r="AN47" s="14" t="n">
         <v>32</v>
       </c>
-      <c r="AL47" s="14" t="n">
+      <c r="AO47" s="14" t="n">
         <v>18</v>
       </c>
-      <c r="AM47" s="14" t="n">
+      <c r="AP47" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="AN47" s="14" t="n">
+      <c r="AQ47" s="14" t="n">
         <v>24</v>
       </c>
-      <c r="AO47" s="15" t="n"/>
+      <c r="AR47" s="15" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="13" t="inlineStr">
@@ -9399,7 +9600,10 @@
       <c r="AL48" s="14" t="n"/>
       <c r="AM48" s="14" t="n"/>
       <c r="AN48" s="14" t="n"/>
-      <c r="AO48" s="15" t="n">
+      <c r="AO48" s="14" t="n"/>
+      <c r="AP48" s="14" t="n"/>
+      <c r="AQ48" s="14" t="n"/>
+      <c r="AR48" s="15" t="n">
         <v>1010</v>
       </c>
     </row>
@@ -9502,7 +9706,10 @@
       <c r="AL49" s="14" t="n"/>
       <c r="AM49" s="14" t="n"/>
       <c r="AN49" s="14" t="n"/>
-      <c r="AO49" s="15" t="n"/>
+      <c r="AO49" s="14" t="n"/>
+      <c r="AP49" s="14" t="n"/>
+      <c r="AQ49" s="14" t="n"/>
+      <c r="AR49" s="15" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="13" t="inlineStr">
@@ -9603,7 +9810,10 @@
       <c r="AL50" s="14" t="n"/>
       <c r="AM50" s="14" t="n"/>
       <c r="AN50" s="14" t="n"/>
-      <c r="AO50" s="15" t="n"/>
+      <c r="AO50" s="14" t="n"/>
+      <c r="AP50" s="14" t="n"/>
+      <c r="AQ50" s="14" t="n"/>
+      <c r="AR50" s="15" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="13" t="inlineStr">
@@ -9704,7 +9914,10 @@
       <c r="AL51" s="14" t="n"/>
       <c r="AM51" s="14" t="n"/>
       <c r="AN51" s="14" t="n"/>
-      <c r="AO51" s="15" t="n"/>
+      <c r="AO51" s="14" t="n"/>
+      <c r="AP51" s="14" t="n"/>
+      <c r="AQ51" s="14" t="n"/>
+      <c r="AR51" s="15" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="13" t="inlineStr">
@@ -9806,16 +10019,19 @@
       <c r="AG52" s="14" t="n"/>
       <c r="AH52" s="14" t="n"/>
       <c r="AI52" s="14" t="n"/>
-      <c r="AJ52" s="14" t="n">
+      <c r="AJ52" s="14" t="n"/>
+      <c r="AK52" s="14" t="n"/>
+      <c r="AL52" s="14" t="n"/>
+      <c r="AM52" s="14" t="n">
         <v>36</v>
       </c>
-      <c r="AK52" s="14" t="n">
+      <c r="AN52" s="14" t="n">
         <v>54</v>
       </c>
-      <c r="AL52" s="14" t="n"/>
-      <c r="AM52" s="14" t="n"/>
-      <c r="AN52" s="14" t="n"/>
-      <c r="AO52" s="15" t="n"/>
+      <c r="AO52" s="14" t="n"/>
+      <c r="AP52" s="14" t="n"/>
+      <c r="AQ52" s="14" t="n"/>
+      <c r="AR52" s="15" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="13" t="inlineStr">
@@ -9921,16 +10137,19 @@
       <c r="AI53" s="14" t="n">
         <v>37.6</v>
       </c>
-      <c r="AJ53" s="14" t="n">
-        <v>25.9</v>
-      </c>
+      <c r="AJ53" s="14" t="n"/>
       <c r="AK53" s="14" t="n"/>
       <c r="AL53" s="14" t="n"/>
       <c r="AM53" s="14" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="AN53" s="14" t="n"/>
+      <c r="AO53" s="14" t="n"/>
+      <c r="AP53" s="14" t="n">
         <v>6.5</v>
       </c>
-      <c r="AN53" s="14" t="n"/>
-      <c r="AO53" s="15" t="n">
+      <c r="AQ53" s="14" t="n"/>
+      <c r="AR53" s="15" t="n">
         <v>245</v>
       </c>
     </row>
@@ -10042,22 +10261,25 @@
       <c r="AI54" s="14" t="n">
         <v>67.67</v>
       </c>
-      <c r="AJ54" s="14" t="n">
+      <c r="AJ54" s="14" t="n"/>
+      <c r="AK54" s="14" t="n"/>
+      <c r="AL54" s="14" t="n"/>
+      <c r="AM54" s="14" t="n">
         <v>29.9</v>
       </c>
-      <c r="AK54" s="14" t="n">
+      <c r="AN54" s="14" t="n">
         <v>29.2</v>
       </c>
-      <c r="AL54" s="14" t="n">
+      <c r="AO54" s="14" t="n">
         <v>17</v>
       </c>
-      <c r="AM54" s="14" t="n">
+      <c r="AP54" s="14" t="n">
         <v>6.75</v>
       </c>
-      <c r="AN54" s="14" t="n">
+      <c r="AQ54" s="14" t="n">
         <v>20.9</v>
       </c>
-      <c r="AO54" s="15" t="n"/>
+      <c r="AR54" s="15" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="13" t="inlineStr">
@@ -10169,22 +10391,25 @@
       <c r="AI55" s="14" t="n">
         <v>84</v>
       </c>
-      <c r="AJ55" s="14" t="n">
+      <c r="AJ55" s="14" t="n"/>
+      <c r="AK55" s="14" t="n"/>
+      <c r="AL55" s="14" t="n"/>
+      <c r="AM55" s="14" t="n">
         <v>45</v>
       </c>
-      <c r="AK55" s="14" t="n">
+      <c r="AN55" s="14" t="n">
         <v>28</v>
       </c>
-      <c r="AL55" s="14" t="n">
+      <c r="AO55" s="14" t="n">
         <v>19</v>
       </c>
-      <c r="AM55" s="14" t="n">
+      <c r="AP55" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="AN55" s="14" t="n">
+      <c r="AQ55" s="14" t="n">
         <v>29</v>
       </c>
-      <c r="AO55" s="15" t="n"/>
+      <c r="AR55" s="15" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="17" t="inlineStr">
@@ -10293,11 +10518,14 @@
       <c r="AJ56" s="18" t="n"/>
       <c r="AK56" s="18" t="n"/>
       <c r="AL56" s="18" t="n"/>
-      <c r="AM56" s="18" t="n">
+      <c r="AM56" s="18" t="n"/>
+      <c r="AN56" s="18" t="n"/>
+      <c r="AO56" s="18" t="n"/>
+      <c r="AP56" s="18" t="n">
         <v>7.5</v>
       </c>
-      <c r="AN56" s="18" t="n"/>
-      <c r="AO56" s="19" t="n">
+      <c r="AQ56" s="18" t="n"/>
+      <c r="AR56" s="19" t="n">
         <v>287</v>
       </c>
     </row>
@@ -10317,7 +10545,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:AO1"/>
+    <mergeCell ref="A1:AR1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10685,7 +10913,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:K32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -11733,7 +11961,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Cesta por pessoa, nível baixo (R$)</t>
+          <t>Consumo por pessoa (bebida + entrada ou prato), nível baixo (R$)</t>
         </is>
       </c>
       <c r="C23" s="4">
@@ -11781,7 +12009,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Cesta por pessoa, nível mediano (R$)</t>
+          <t>Consumo por pessoa (bebida + entrada ou prato), nível mediano (R$)</t>
         </is>
       </c>
       <c r="C24" s="4">
@@ -11829,7 +12057,7 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Cesta por pessoa, nível alto (R$)</t>
+          <t>Consumo por pessoa (bebida + entrada ou prato), nível alto (R$)</t>
         </is>
       </c>
       <c r="C25" s="4">
@@ -11870,69 +12098,213 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="inlineStr">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Cardápio</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Cesta completa (consumo + couvert encontrado), nível baixo (R$)</t>
+        </is>
+      </c>
+      <c r="C26" s="4">
+        <f>COUNT('Dados B1'!$AJ$3:$AJ$56)</f>
+        <v/>
+      </c>
+      <c r="D26" s="4">
+        <f>ROWS('Dados B1'!$AJ$3:$AJ$56)-COUNT('Dados B1'!$AJ$3:$AJ$56)</f>
+        <v/>
+      </c>
+      <c r="E26" s="10">
+        <f>IFERROR(AVERAGE('Dados B1'!$AJ$3:$AJ$56),"")</f>
+        <v/>
+      </c>
+      <c r="F26" s="10">
+        <f>IFERROR(MEDIAN('Dados B1'!$AJ$3:$AJ$56),"")</f>
+        <v/>
+      </c>
+      <c r="G26" s="10">
+        <f>IFERROR(STDEV('Dados B1'!$AJ$3:$AJ$56),"")</f>
+        <v/>
+      </c>
+      <c r="H26" s="10">
+        <f>IFERROR(MIN('Dados B1'!$AJ$3:$AJ$56),"")</f>
+        <v/>
+      </c>
+      <c r="I26" s="10">
+        <f>IFERROR(PERCENTILE('Dados B1'!$AJ$3:$AJ$56,0.25),"")</f>
+        <v/>
+      </c>
+      <c r="J26" s="10">
+        <f>IFERROR(PERCENTILE('Dados B1'!$AJ$3:$AJ$56,0.75),"")</f>
+        <v/>
+      </c>
+      <c r="K26" s="10">
+        <f>IFERROR(MAX('Dados B1'!$AJ$3:$AJ$56),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Cardápio</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Cesta completa (consumo + couvert encontrado), nível mediano (R$)</t>
+        </is>
+      </c>
+      <c r="C27" s="4">
+        <f>COUNT('Dados B1'!$AK$3:$AK$56)</f>
+        <v/>
+      </c>
+      <c r="D27" s="4">
+        <f>ROWS('Dados B1'!$AK$3:$AK$56)-COUNT('Dados B1'!$AK$3:$AK$56)</f>
+        <v/>
+      </c>
+      <c r="E27" s="10">
+        <f>IFERROR(AVERAGE('Dados B1'!$AK$3:$AK$56),"")</f>
+        <v/>
+      </c>
+      <c r="F27" s="10">
+        <f>IFERROR(MEDIAN('Dados B1'!$AK$3:$AK$56),"")</f>
+        <v/>
+      </c>
+      <c r="G27" s="10">
+        <f>IFERROR(STDEV('Dados B1'!$AK$3:$AK$56),"")</f>
+        <v/>
+      </c>
+      <c r="H27" s="10">
+        <f>IFERROR(MIN('Dados B1'!$AK$3:$AK$56),"")</f>
+        <v/>
+      </c>
+      <c r="I27" s="10">
+        <f>IFERROR(PERCENTILE('Dados B1'!$AK$3:$AK$56,0.25),"")</f>
+        <v/>
+      </c>
+      <c r="J27" s="10">
+        <f>IFERROR(PERCENTILE('Dados B1'!$AK$3:$AK$56,0.75),"")</f>
+        <v/>
+      </c>
+      <c r="K27" s="10">
+        <f>IFERROR(MAX('Dados B1'!$AK$3:$AK$56),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Cardápio</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Cesta completa (consumo + couvert encontrado), nível alto (R$)</t>
+        </is>
+      </c>
+      <c r="C28" s="4">
+        <f>COUNT('Dados B1'!$AL$3:$AL$56)</f>
+        <v/>
+      </c>
+      <c r="D28" s="4">
+        <f>ROWS('Dados B1'!$AL$3:$AL$56)-COUNT('Dados B1'!$AL$3:$AL$56)</f>
+        <v/>
+      </c>
+      <c r="E28" s="10">
+        <f>IFERROR(AVERAGE('Dados B1'!$AL$3:$AL$56),"")</f>
+        <v/>
+      </c>
+      <c r="F28" s="10">
+        <f>IFERROR(MEDIAN('Dados B1'!$AL$3:$AL$56),"")</f>
+        <v/>
+      </c>
+      <c r="G28" s="10">
+        <f>IFERROR(STDEV('Dados B1'!$AL$3:$AL$56),"")</f>
+        <v/>
+      </c>
+      <c r="H28" s="10">
+        <f>IFERROR(MIN('Dados B1'!$AL$3:$AL$56),"")</f>
+        <v/>
+      </c>
+      <c r="I28" s="10">
+        <f>IFERROR(PERCENTILE('Dados B1'!$AL$3:$AL$56,0.25),"")</f>
+        <v/>
+      </c>
+      <c r="J28" s="10">
+        <f>IFERROR(PERCENTILE('Dados B1'!$AL$3:$AL$56,0.75),"")</f>
+        <v/>
+      </c>
+      <c r="K28" s="10">
+        <f>IFERROR(MAX('Dados B1'!$AL$3:$AL$56),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
         <is>
           <t>Acervo</t>
         </is>
       </c>
-      <c r="B26" s="6" t="inlineStr">
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>Títulos no acervo publicado</t>
         </is>
       </c>
-      <c r="C26" s="7">
-        <f>COUNT('Dados B1'!$AO$3:$AO$56)</f>
-        <v/>
-      </c>
-      <c r="D26" s="7">
-        <f>ROWS('Dados B1'!$AO$3:$AO$56)-COUNT('Dados B1'!$AO$3:$AO$56)</f>
-        <v/>
-      </c>
-      <c r="E26" s="11">
-        <f>IFERROR(AVERAGE('Dados B1'!$AO$3:$AO$56),"")</f>
-        <v/>
-      </c>
-      <c r="F26" s="11">
-        <f>IFERROR(MEDIAN('Dados B1'!$AO$3:$AO$56),"")</f>
-        <v/>
-      </c>
-      <c r="G26" s="11">
-        <f>IFERROR(STDEV('Dados B1'!$AO$3:$AO$56),"")</f>
-        <v/>
-      </c>
-      <c r="H26" s="11">
-        <f>IFERROR(MIN('Dados B1'!$AO$3:$AO$56),"")</f>
-        <v/>
-      </c>
-      <c r="I26" s="11">
-        <f>IFERROR(PERCENTILE('Dados B1'!$AO$3:$AO$56,0.25),"")</f>
-        <v/>
-      </c>
-      <c r="J26" s="11">
-        <f>IFERROR(PERCENTILE('Dados B1'!$AO$3:$AO$56,0.75),"")</f>
-        <v/>
-      </c>
-      <c r="K26" s="11">
-        <f>IFERROR(MAX('Dados B1'!$AO$3:$AO$56),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="9" t="inlineStr">
+      <c r="C29" s="7">
+        <f>COUNT('Dados B1'!$AR$3:$AR$56)</f>
+        <v/>
+      </c>
+      <c r="D29" s="7">
+        <f>ROWS('Dados B1'!$AR$3:$AR$56)-COUNT('Dados B1'!$AR$3:$AR$56)</f>
+        <v/>
+      </c>
+      <c r="E29" s="11">
+        <f>IFERROR(AVERAGE('Dados B1'!$AR$3:$AR$56),"")</f>
+        <v/>
+      </c>
+      <c r="F29" s="11">
+        <f>IFERROR(MEDIAN('Dados B1'!$AR$3:$AR$56),"")</f>
+        <v/>
+      </c>
+      <c r="G29" s="11">
+        <f>IFERROR(STDEV('Dados B1'!$AR$3:$AR$56),"")</f>
+        <v/>
+      </c>
+      <c r="H29" s="11">
+        <f>IFERROR(MIN('Dados B1'!$AR$3:$AR$56),"")</f>
+        <v/>
+      </c>
+      <c r="I29" s="11">
+        <f>IFERROR(PERCENTILE('Dados B1'!$AR$3:$AR$56,0.25),"")</f>
+        <v/>
+      </c>
+      <c r="J29" s="11">
+        <f>IFERROR(PERCENTILE('Dados B1'!$AR$3:$AR$56,0.75),"")</f>
+        <v/>
+      </c>
+      <c r="K29" s="11">
+        <f>IFERROR(MAX('Dados B1'!$AR$3:$AR$56),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
         <is>
           <t>Fonte: B1, Google Places API (09/2026 e 15/10/2026), coletor de entorno do Google Maps (15/10/2026), Instagram (01/09 a 01/10/2026) e cardápios</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="9" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="9" t="inlineStr">
         <is>
           <t>Nota: desvio padrão amostral; quartis pelo método inclusivo. Engajamento em fração (0,01 = 1%).</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="9" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
         <is>
           <t>Entorno sem OpenStreetMap: shoppings de porte fora. Distância ao metrô vazia onde a cidade não tem metrô lido (Curitiba, Florianópolis, Belém, Goiânia, Vitória).</t>
         </is>
@@ -12152,7 +12524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -12165,6 +12537,8 @@
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -12217,12 +12591,22 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>casas com cesta</t>
+          <t>casas com consumo</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>cesta mediana (mediana, R$)</t>
+          <t>consumo mediano (mediana, R$)</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>casas com cesta completa</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>cesta completa mediana (mediana, R$)</t>
         </is>
       </c>
     </row>
@@ -12268,6 +12652,14 @@
         <f t="array" ref="J3">IFERROR(MEDIAN(IF('Dados B1'!$C$3:$C$56=$A3,IF('Dados B1'!$AH$3:$AH$56&lt;&gt;"",'Dados B1'!$AH$3:$AH$56))),"")</f>
         <v/>
       </c>
+      <c r="K3" s="4">
+        <f>COUNTIFS('Dados B1'!$C$3:$C$56,$A3,'Dados B1'!$AK$3:$AK$56,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="L3" s="10">
+        <f t="array" ref="L3">IFERROR(MEDIAN(IF('Dados B1'!$C$3:$C$56=$A3,IF('Dados B1'!$AK$3:$AK$56&lt;&gt;"",'Dados B1'!$AK$3:$AK$56))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -12311,6 +12703,14 @@
         <f t="array" ref="J4">IFERROR(MEDIAN(IF('Dados B1'!$C$3:$C$56=$A4,IF('Dados B1'!$AH$3:$AH$56&lt;&gt;"",'Dados B1'!$AH$3:$AH$56))),"")</f>
         <v/>
       </c>
+      <c r="K4" s="4">
+        <f>COUNTIFS('Dados B1'!$C$3:$C$56,$A4,'Dados B1'!$AK$3:$AK$56,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="L4" s="10">
+        <f t="array" ref="L4">IFERROR(MEDIAN(IF('Dados B1'!$C$3:$C$56=$A4,IF('Dados B1'!$AK$3:$AK$56&lt;&gt;"",'Dados B1'!$AK$3:$AK$56))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -12354,6 +12754,14 @@
         <f t="array" ref="J5">IFERROR(MEDIAN(IF('Dados B1'!$C$3:$C$56=$A5,IF('Dados B1'!$AH$3:$AH$56&lt;&gt;"",'Dados B1'!$AH$3:$AH$56))),"")</f>
         <v/>
       </c>
+      <c r="K5" s="4">
+        <f>COUNTIFS('Dados B1'!$C$3:$C$56,$A5,'Dados B1'!$AK$3:$AK$56,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="L5" s="10">
+        <f t="array" ref="L5">IFERROR(MEDIAN(IF('Dados B1'!$C$3:$C$56=$A5,IF('Dados B1'!$AK$3:$AK$56&lt;&gt;"",'Dados B1'!$AK$3:$AK$56))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -12397,6 +12805,14 @@
         <f t="array" ref="J6">IFERROR(MEDIAN(IF('Dados B1'!$C$3:$C$56=$A6,IF('Dados B1'!$AH$3:$AH$56&lt;&gt;"",'Dados B1'!$AH$3:$AH$56))),"")</f>
         <v/>
       </c>
+      <c r="K6" s="4">
+        <f>COUNTIFS('Dados B1'!$C$3:$C$56,$A6,'Dados B1'!$AK$3:$AK$56,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="L6" s="10">
+        <f t="array" ref="L6">IFERROR(MEDIAN(IF('Dados B1'!$C$3:$C$56=$A6,IF('Dados B1'!$AK$3:$AK$56&lt;&gt;"",'Dados B1'!$AK$3:$AK$56))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -12440,6 +12856,14 @@
         <f t="array" ref="J7">IFERROR(MEDIAN(IF('Dados B1'!$C$3:$C$56=$A7,IF('Dados B1'!$AH$3:$AH$56&lt;&gt;"",'Dados B1'!$AH$3:$AH$56))),"")</f>
         <v/>
       </c>
+      <c r="K7" s="4">
+        <f>COUNTIFS('Dados B1'!$C$3:$C$56,$A7,'Dados B1'!$AK$3:$AK$56,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="L7" s="10">
+        <f t="array" ref="L7">IFERROR(MEDIAN(IF('Dados B1'!$C$3:$C$56=$A7,IF('Dados B1'!$AK$3:$AK$56&lt;&gt;"",'Dados B1'!$AK$3:$AK$56))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -12483,6 +12907,14 @@
         <f>MEDIAN('Dados B1'!$AH$3:$AH$56)</f>
         <v/>
       </c>
+      <c r="K8" s="7">
+        <f>COUNT('Dados B1'!$AK$3:$AK$56)</f>
+        <v/>
+      </c>
+      <c r="L8" s="11">
+        <f>MEDIAN('Dados B1'!$AK$3:$AK$56)</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -12494,13 +12926,13 @@
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>Nota: medianas calculadas só entre as casas com dado; cesta só nas casas com couvert, bebida e prato encontrados.</t>
+          <t>Nota: medianas calculadas só entre as casas com dado. Consumo = bebida + entrada ou prato, nas casas com os dois no cardápio; cesta completa = consumo + couvert, só nas casas com couvert encontrado (couvert não encontrado não entra como 0).</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A1:L1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -12513,7 +12945,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -12527,6 +12959,8 @@
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -12584,12 +13018,22 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>casas com cesta</t>
+          <t>casas com consumo</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>cesta mediana (mediana, R$)</t>
+          <t>consumo mediano (mediana, R$)</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>casas com cesta completa</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>cesta completa mediana (mediana, R$)</t>
         </is>
       </c>
     </row>
@@ -12640,6 +13084,14 @@
         <f t="array" ref="K3">IFERROR(MEDIAN(IF('Dados B1'!$B$3:$B$56=$A3,IF('Dados B1'!$AH$3:$AH$56&lt;&gt;"",'Dados B1'!$AH$3:$AH$56))),"")</f>
         <v/>
       </c>
+      <c r="L3" s="4">
+        <f>COUNTIFS('Dados B1'!$B$3:$B$56,$A3,'Dados B1'!$AK$3:$AK$56,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="M3" s="10">
+        <f t="array" ref="M3">IFERROR(MEDIAN(IF('Dados B1'!$B$3:$B$56=$A3,IF('Dados B1'!$AK$3:$AK$56&lt;&gt;"",'Dados B1'!$AK$3:$AK$56))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -12688,6 +13140,14 @@
         <f t="array" ref="K4">IFERROR(MEDIAN(IF('Dados B1'!$B$3:$B$56=$A4,IF('Dados B1'!$AH$3:$AH$56&lt;&gt;"",'Dados B1'!$AH$3:$AH$56))),"")</f>
         <v/>
       </c>
+      <c r="L4" s="4">
+        <f>COUNTIFS('Dados B1'!$B$3:$B$56,$A4,'Dados B1'!$AK$3:$AK$56,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="M4" s="10">
+        <f t="array" ref="M4">IFERROR(MEDIAN(IF('Dados B1'!$B$3:$B$56=$A4,IF('Dados B1'!$AK$3:$AK$56&lt;&gt;"",'Dados B1'!$AK$3:$AK$56))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -12736,6 +13196,14 @@
         <f t="array" ref="K5">IFERROR(MEDIAN(IF('Dados B1'!$B$3:$B$56=$A5,IF('Dados B1'!$AH$3:$AH$56&lt;&gt;"",'Dados B1'!$AH$3:$AH$56))),"")</f>
         <v/>
       </c>
+      <c r="L5" s="4">
+        <f>COUNTIFS('Dados B1'!$B$3:$B$56,$A5,'Dados B1'!$AK$3:$AK$56,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="M5" s="10">
+        <f t="array" ref="M5">IFERROR(MEDIAN(IF('Dados B1'!$B$3:$B$56=$A5,IF('Dados B1'!$AK$3:$AK$56&lt;&gt;"",'Dados B1'!$AK$3:$AK$56))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -12784,6 +13252,14 @@
         <f t="array" ref="K6">IFERROR(MEDIAN(IF('Dados B1'!$B$3:$B$56=$A6,IF('Dados B1'!$AH$3:$AH$56&lt;&gt;"",'Dados B1'!$AH$3:$AH$56))),"")</f>
         <v/>
       </c>
+      <c r="L6" s="4">
+        <f>COUNTIFS('Dados B1'!$B$3:$B$56,$A6,'Dados B1'!$AK$3:$AK$56,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="M6" s="10">
+        <f t="array" ref="M6">IFERROR(MEDIAN(IF('Dados B1'!$B$3:$B$56=$A6,IF('Dados B1'!$AK$3:$AK$56&lt;&gt;"",'Dados B1'!$AK$3:$AK$56))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -12832,6 +13308,14 @@
         <f t="array" ref="K7">IFERROR(MEDIAN(IF('Dados B1'!$B$3:$B$56=$A7,IF('Dados B1'!$AH$3:$AH$56&lt;&gt;"",'Dados B1'!$AH$3:$AH$56))),"")</f>
         <v/>
       </c>
+      <c r="L7" s="4">
+        <f>COUNTIFS('Dados B1'!$B$3:$B$56,$A7,'Dados B1'!$AK$3:$AK$56,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="M7" s="10">
+        <f t="array" ref="M7">IFERROR(MEDIAN(IF('Dados B1'!$B$3:$B$56=$A7,IF('Dados B1'!$AK$3:$AK$56&lt;&gt;"",'Dados B1'!$AK$3:$AK$56))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -12880,6 +13364,14 @@
         <f t="array" ref="K8">IFERROR(MEDIAN(IF('Dados B1'!$B$3:$B$56=$A8,IF('Dados B1'!$AH$3:$AH$56&lt;&gt;"",'Dados B1'!$AH$3:$AH$56))),"")</f>
         <v/>
       </c>
+      <c r="L8" s="4">
+        <f>COUNTIFS('Dados B1'!$B$3:$B$56,$A8,'Dados B1'!$AK$3:$AK$56,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="M8" s="10">
+        <f t="array" ref="M8">IFERROR(MEDIAN(IF('Dados B1'!$B$3:$B$56=$A8,IF('Dados B1'!$AK$3:$AK$56&lt;&gt;"",'Dados B1'!$AK$3:$AK$56))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -12928,6 +13420,14 @@
         <f t="array" ref="K9">IFERROR(MEDIAN(IF('Dados B1'!$B$3:$B$56=$A9,IF('Dados B1'!$AH$3:$AH$56&lt;&gt;"",'Dados B1'!$AH$3:$AH$56))),"")</f>
         <v/>
       </c>
+      <c r="L9" s="4">
+        <f>COUNTIFS('Dados B1'!$B$3:$B$56,$A9,'Dados B1'!$AK$3:$AK$56,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="M9" s="10">
+        <f t="array" ref="M9">IFERROR(MEDIAN(IF('Dados B1'!$B$3:$B$56=$A9,IF('Dados B1'!$AK$3:$AK$56&lt;&gt;"",'Dados B1'!$AK$3:$AK$56))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -12976,6 +13476,14 @@
         <f t="array" ref="K10">IFERROR(MEDIAN(IF('Dados B1'!$B$3:$B$56=$A10,IF('Dados B1'!$AH$3:$AH$56&lt;&gt;"",'Dados B1'!$AH$3:$AH$56))),"")</f>
         <v/>
       </c>
+      <c r="L10" s="4">
+        <f>COUNTIFS('Dados B1'!$B$3:$B$56,$A10,'Dados B1'!$AK$3:$AK$56,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="M10" s="10">
+        <f t="array" ref="M10">IFERROR(MEDIAN(IF('Dados B1'!$B$3:$B$56=$A10,IF('Dados B1'!$AK$3:$AK$56&lt;&gt;"",'Dados B1'!$AK$3:$AK$56))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -13024,6 +13532,14 @@
         <f t="array" ref="K11">IFERROR(MEDIAN(IF('Dados B1'!$B$3:$B$56=$A11,IF('Dados B1'!$AH$3:$AH$56&lt;&gt;"",'Dados B1'!$AH$3:$AH$56))),"")</f>
         <v/>
       </c>
+      <c r="L11" s="4">
+        <f>COUNTIFS('Dados B1'!$B$3:$B$56,$A11,'Dados B1'!$AK$3:$AK$56,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="M11" s="10">
+        <f t="array" ref="M11">IFERROR(MEDIAN(IF('Dados B1'!$B$3:$B$56=$A11,IF('Dados B1'!$AK$3:$AK$56&lt;&gt;"",'Dados B1'!$AK$3:$AK$56))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -13072,6 +13588,14 @@
         <f t="array" ref="K12">IFERROR(MEDIAN(IF('Dados B1'!$B$3:$B$56=$A12,IF('Dados B1'!$AH$3:$AH$56&lt;&gt;"",'Dados B1'!$AH$3:$AH$56))),"")</f>
         <v/>
       </c>
+      <c r="L12" s="4">
+        <f>COUNTIFS('Dados B1'!$B$3:$B$56,$A12,'Dados B1'!$AK$3:$AK$56,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="M12" s="10">
+        <f t="array" ref="M12">IFERROR(MEDIAN(IF('Dados B1'!$B$3:$B$56=$A12,IF('Dados B1'!$AK$3:$AK$56&lt;&gt;"",'Dados B1'!$AK$3:$AK$56))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -13120,6 +13644,14 @@
         <f t="array" ref="K13">IFERROR(MEDIAN(IF('Dados B1'!$B$3:$B$56=$A13,IF('Dados B1'!$AH$3:$AH$56&lt;&gt;"",'Dados B1'!$AH$3:$AH$56))),"")</f>
         <v/>
       </c>
+      <c r="L13" s="4">
+        <f>COUNTIFS('Dados B1'!$B$3:$B$56,$A13,'Dados B1'!$AK$3:$AK$56,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="M13" s="10">
+        <f t="array" ref="M13">IFERROR(MEDIAN(IF('Dados B1'!$B$3:$B$56=$A13,IF('Dados B1'!$AK$3:$AK$56&lt;&gt;"",'Dados B1'!$AK$3:$AK$56))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -13168,6 +13700,14 @@
         <f t="array" ref="K14">IFERROR(MEDIAN(IF('Dados B1'!$B$3:$B$56=$A14,IF('Dados B1'!$AH$3:$AH$56&lt;&gt;"",'Dados B1'!$AH$3:$AH$56))),"")</f>
         <v/>
       </c>
+      <c r="L14" s="4">
+        <f>COUNTIFS('Dados B1'!$B$3:$B$56,$A14,'Dados B1'!$AK$3:$AK$56,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="M14" s="10">
+        <f t="array" ref="M14">IFERROR(MEDIAN(IF('Dados B1'!$B$3:$B$56=$A14,IF('Dados B1'!$AK$3:$AK$56&lt;&gt;"",'Dados B1'!$AK$3:$AK$56))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -13214,6 +13754,14 @@
       </c>
       <c r="K15" s="10">
         <f t="array" ref="K15">IFERROR(MEDIAN(IF('Dados B1'!$B$3:$B$56=$A15,IF('Dados B1'!$AH$3:$AH$56&lt;&gt;"",'Dados B1'!$AH$3:$AH$56))),"")</f>
+        <v/>
+      </c>
+      <c r="L15" s="4">
+        <f>COUNTIFS('Dados B1'!$B$3:$B$56,$A15,'Dados B1'!$AK$3:$AK$56,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="M15" s="10">
+        <f t="array" ref="M15">IFERROR(MEDIAN(IF('Dados B1'!$B$3:$B$56=$A15,IF('Dados B1'!$AK$3:$AK$56&lt;&gt;"",'Dados B1'!$AK$3:$AK$56))),"")</f>
         <v/>
       </c>
     </row>
@@ -13260,6 +13808,14 @@
         <f>MEDIAN('Dados B1'!$AH$3:$AH$56)</f>
         <v/>
       </c>
+      <c r="L16" s="7">
+        <f>COUNT('Dados B1'!$AK$3:$AK$56)</f>
+        <v/>
+      </c>
+      <c r="M16" s="11">
+        <f>MEDIAN('Dados B1'!$AK$3:$AK$56)</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
@@ -13271,13 +13827,20 @@
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>Nota: o gráfico mostra a mediana da cesta mediana das casas com cesta em cada metrópole; metrópoles sem cesta ficam fora.</t>
+          <t>Nota: o gráfico mostra a mediana do consumo mediano das casas com consumo em cada metrópole; metrópoles sem consumo ficam fora.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>Consumo = bebida + entrada ou prato, nas casas com os dois no cardápio; cesta completa = consumo + couvert, só nas casas com couvert encontrado (couvert não encontrado não entra como 0).</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -13518,7 +14081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -13638,19 +14201,19 @@
         </is>
       </c>
       <c r="B6" s="4">
-        <f>COUNT('Dados B1'!$AJ$3:$AJ$56)</f>
+        <f>COUNT('Dados B1'!$AM$3:$AM$56)</f>
         <v/>
       </c>
       <c r="C6" s="10">
-        <f>IFERROR(PERCENTILE('Dados B1'!$AJ$3:$AJ$56,0.25),"")</f>
+        <f>IFERROR(PERCENTILE('Dados B1'!$AM$3:$AM$56,0.25),"")</f>
         <v/>
       </c>
       <c r="D6" s="10">
-        <f>IFERROR(MEDIAN('Dados B1'!$AJ$3:$AJ$56),"")</f>
+        <f>IFERROR(MEDIAN('Dados B1'!$AM$3:$AM$56),"")</f>
         <v/>
       </c>
       <c r="E6" s="10">
-        <f>IFERROR(PERCENTILE('Dados B1'!$AJ$3:$AJ$56,0.75),"")</f>
+        <f>IFERROR(PERCENTILE('Dados B1'!$AM$3:$AM$56,0.75),"")</f>
         <v/>
       </c>
     </row>
@@ -13661,19 +14224,19 @@
         </is>
       </c>
       <c r="B7" s="4">
-        <f>COUNT('Dados B1'!$AK$3:$AK$56)</f>
+        <f>COUNT('Dados B1'!$AN$3:$AN$56)</f>
         <v/>
       </c>
       <c r="C7" s="10">
-        <f>IFERROR(PERCENTILE('Dados B1'!$AK$3:$AK$56,0.25),"")</f>
+        <f>IFERROR(PERCENTILE('Dados B1'!$AN$3:$AN$56,0.25),"")</f>
         <v/>
       </c>
       <c r="D7" s="10">
-        <f>IFERROR(MEDIAN('Dados B1'!$AK$3:$AK$56),"")</f>
+        <f>IFERROR(MEDIAN('Dados B1'!$AN$3:$AN$56),"")</f>
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>IFERROR(PERCENTILE('Dados B1'!$AK$3:$AK$56,0.75),"")</f>
+        <f>IFERROR(PERCENTILE('Dados B1'!$AN$3:$AN$56,0.75),"")</f>
         <v/>
       </c>
     </row>
@@ -13684,19 +14247,19 @@
         </is>
       </c>
       <c r="B8" s="4">
-        <f>COUNT('Dados B1'!$AL$3:$AL$56)</f>
+        <f>COUNT('Dados B1'!$AO$3:$AO$56)</f>
         <v/>
       </c>
       <c r="C8" s="10">
-        <f>IFERROR(PERCENTILE('Dados B1'!$AL$3:$AL$56,0.25),"")</f>
+        <f>IFERROR(PERCENTILE('Dados B1'!$AO$3:$AO$56,0.25),"")</f>
         <v/>
       </c>
       <c r="D8" s="10">
-        <f>IFERROR(MEDIAN('Dados B1'!$AL$3:$AL$56),"")</f>
+        <f>IFERROR(MEDIAN('Dados B1'!$AO$3:$AO$56),"")</f>
         <v/>
       </c>
       <c r="E8" s="10">
-        <f>IFERROR(PERCENTILE('Dados B1'!$AL$3:$AL$56,0.75),"")</f>
+        <f>IFERROR(PERCENTILE('Dados B1'!$AO$3:$AO$56,0.75),"")</f>
         <v/>
       </c>
     </row>
@@ -13707,19 +14270,19 @@
         </is>
       </c>
       <c r="B9" s="4">
-        <f>COUNT('Dados B1'!$AM$3:$AM$56)</f>
+        <f>COUNT('Dados B1'!$AP$3:$AP$56)</f>
         <v/>
       </c>
       <c r="C9" s="10">
-        <f>IFERROR(PERCENTILE('Dados B1'!$AM$3:$AM$56,0.25),"")</f>
+        <f>IFERROR(PERCENTILE('Dados B1'!$AP$3:$AP$56,0.25),"")</f>
         <v/>
       </c>
       <c r="D9" s="10">
-        <f>IFERROR(MEDIAN('Dados B1'!$AM$3:$AM$56),"")</f>
+        <f>IFERROR(MEDIAN('Dados B1'!$AP$3:$AP$56),"")</f>
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>IFERROR(PERCENTILE('Dados B1'!$AM$3:$AM$56,0.75),"")</f>
+        <f>IFERROR(PERCENTILE('Dados B1'!$AP$3:$AP$56,0.75),"")</f>
         <v/>
       </c>
     </row>
@@ -13730,26 +14293,26 @@
         </is>
       </c>
       <c r="B10" s="4">
-        <f>COUNT('Dados B1'!$AN$3:$AN$56)</f>
+        <f>COUNT('Dados B1'!$AQ$3:$AQ$56)</f>
         <v/>
       </c>
       <c r="C10" s="10">
-        <f>IFERROR(PERCENTILE('Dados B1'!$AN$3:$AN$56,0.25),"")</f>
+        <f>IFERROR(PERCENTILE('Dados B1'!$AQ$3:$AQ$56,0.25),"")</f>
         <v/>
       </c>
       <c r="D10" s="10">
-        <f>IFERROR(MEDIAN('Dados B1'!$AN$3:$AN$56),"")</f>
+        <f>IFERROR(MEDIAN('Dados B1'!$AQ$3:$AQ$56),"")</f>
         <v/>
       </c>
       <c r="E10" s="10">
-        <f>IFERROR(PERCENTILE('Dados B1'!$AN$3:$AN$56,0.75),"")</f>
+        <f>IFERROR(PERCENTILE('Dados B1'!$AQ$3:$AQ$56,0.75),"")</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Cesta por pessoa, nível baixo</t>
+          <t>Consumo por pessoa, nível baixo</t>
         </is>
       </c>
       <c r="B11" s="4">
@@ -13772,7 +14335,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Cesta por pessoa, nível mediano</t>
+          <t>Consumo por pessoa, nível mediano</t>
         </is>
       </c>
       <c r="B12" s="4">
@@ -13793,46 +14356,115 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>Cesta por pessoa, nível alto</t>
-        </is>
-      </c>
-      <c r="B13" s="7">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Consumo por pessoa, nível alto</t>
+        </is>
+      </c>
+      <c r="B13" s="4">
         <f>COUNT('Dados B1'!$AI$3:$AI$56)</f>
         <v/>
       </c>
-      <c r="C13" s="11">
+      <c r="C13" s="10">
         <f>IFERROR(PERCENTILE('Dados B1'!$AI$3:$AI$56,0.25),"")</f>
         <v/>
       </c>
-      <c r="D13" s="11">
+      <c r="D13" s="10">
         <f>IFERROR(MEDIAN('Dados B1'!$AI$3:$AI$56),"")</f>
         <v/>
       </c>
-      <c r="E13" s="11">
+      <c r="E13" s="10">
         <f>IFERROR(PERCENTILE('Dados B1'!$AI$3:$AI$56,0.75),"")</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Cesta completa, nível baixo</t>
+        </is>
+      </c>
+      <c r="B14" s="4">
+        <f>COUNT('Dados B1'!$AJ$3:$AJ$56)</f>
+        <v/>
+      </c>
+      <c r="C14" s="10">
+        <f>IFERROR(PERCENTILE('Dados B1'!$AJ$3:$AJ$56,0.25),"")</f>
+        <v/>
+      </c>
+      <c r="D14" s="10">
+        <f>IFERROR(MEDIAN('Dados B1'!$AJ$3:$AJ$56),"")</f>
+        <v/>
+      </c>
+      <c r="E14" s="10">
+        <f>IFERROR(PERCENTILE('Dados B1'!$AJ$3:$AJ$56,0.75),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Cesta completa, nível mediano</t>
+        </is>
+      </c>
+      <c r="B15" s="4">
+        <f>COUNT('Dados B1'!$AK$3:$AK$56)</f>
+        <v/>
+      </c>
+      <c r="C15" s="10">
+        <f>IFERROR(PERCENTILE('Dados B1'!$AK$3:$AK$56,0.25),"")</f>
+        <v/>
+      </c>
+      <c r="D15" s="10">
+        <f>IFERROR(MEDIAN('Dados B1'!$AK$3:$AK$56),"")</f>
+        <v/>
+      </c>
+      <c r="E15" s="10">
+        <f>IFERROR(PERCENTILE('Dados B1'!$AK$3:$AK$56,0.75),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Cesta completa, nível alto</t>
+        </is>
+      </c>
+      <c r="B16" s="7">
+        <f>COUNT('Dados B1'!$AL$3:$AL$56)</f>
+        <v/>
+      </c>
+      <c r="C16" s="11">
+        <f>IFERROR(PERCENTILE('Dados B1'!$AL$3:$AL$56,0.25),"")</f>
+        <v/>
+      </c>
+      <c r="D16" s="11">
+        <f>IFERROR(MEDIAN('Dados B1'!$AL$3:$AL$56),"")</f>
+        <v/>
+      </c>
+      <c r="E16" s="11">
+        <f>IFERROR(PERCENTILE('Dados B1'!$AL$3:$AL$56,0.75),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>Fonte: B1, cardápios transcritos (B1_cardapios_itens_precos.xlsx)</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="9" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>Nota: cada casa entra com a mediana do próprio cardápio na categoria; quartis entre as casas.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t>Cesta = couvert + bebida + entrada ou prato, só nas casas em que os três foram encontrados.</t>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>Consumo = bebida + entrada ou prato, nas casas com os dois no cardápio; cesta completa = consumo + couvert, só nas casas com couvert encontrado (couvert não encontrado não entra como 0).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
B1: base de cardápios e estatística descritiva regeradas com a main unificada
Depois do PR #22 (branch do Mac + main antiga + app 2.5 + PRs #20 e #21),
as saídas do B1, a planilha agregada e o modelo financeiro foram regeradas
para refletir a base unificada: 42 cardápios, consumo por pessoa em 36 casas
(mediana R$ 50,25), cesta completa em 10 (R$ 78,50), couvert em 13 (R$ 20,00).
Somas por metrópole, região e capital fecham com 54 casas.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/Dados agregados/B1_dados_agregados_completo.xlsx
+++ b/dados/Dados agregados/B1_dados_agregados_completo.xlsx
@@ -1,28 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Índice" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tab 1" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tab 2" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tab 3" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tab 4" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tab 5" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tab 6" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tab 7" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tab 8" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tab 9" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tab 10" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tab 11" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tab 12" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tab 13" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tab 14" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados B1" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Índice" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Tab 1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Tab 2" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Tab 3" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Tab 4" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Tab 5" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Tab 6" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Tab 7" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Tab 8" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Tab 9" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Tab 10" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Tab 11" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Tab 12" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Tab 13" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Tab 14" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Dados B1" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -266,7 +266,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>5</col>
@@ -274,21 +274,21 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5905500" cy="3469613"/>
+    <ext cx="5905500" cy="3395274"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:prstGeom prst="rect"/>
+        <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -299,7 +299,7 @@
 </file>
 
 <file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>8</col>
@@ -307,21 +307,21 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5905500" cy="3462849"/>
+    <ext cx="5905500" cy="3463245"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:prstGeom prst="rect"/>
+        <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -332,7 +332,7 @@
 </file>
 
 <file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>7</col>
@@ -340,21 +340,21 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5905500" cy="4575140"/>
+    <ext cx="5905500" cy="4384218"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:prstGeom prst="rect"/>
+        <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -365,7 +365,7 @@
 </file>
 
 <file path=xl/drawings/drawing12.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>8</col>
@@ -373,21 +373,21 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5905500" cy="4481896"/>
+    <ext cx="5905500" cy="4346543"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:prstGeom prst="rect"/>
+        <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -398,7 +398,7 @@
 </file>
 
 <file path=xl/drawings/drawing13.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>8</col>
@@ -406,21 +406,21 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5905500" cy="2357882"/>
+    <ext cx="5905500" cy="2281460"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:prstGeom prst="rect"/>
+        <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -431,7 +431,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>5</col>
@@ -439,21 +439,21 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5905500" cy="3121190"/>
+    <ext cx="5905500" cy="3111469"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:prstGeom prst="rect"/>
+        <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -464,7 +464,7 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>13</col>
@@ -472,21 +472,21 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5905500" cy="3602946"/>
+    <ext cx="5905500" cy="3540146"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:prstGeom prst="rect"/>
+        <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -497,7 +497,7 @@
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>14</col>
@@ -505,21 +505,21 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5905500" cy="3263218"/>
+    <ext cx="5905500" cy="3188403"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:prstGeom prst="rect"/>
+        <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -530,7 +530,7 @@
 </file>
 
 <file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>6</col>
@@ -538,21 +538,21 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5905500" cy="2120488"/>
+    <ext cx="5905500" cy="1955047"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:prstGeom prst="rect"/>
+        <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -563,7 +563,7 @@
 </file>
 
 <file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>6</col>
@@ -571,21 +571,21 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5905500" cy="3295926"/>
+    <ext cx="5905500" cy="3183595"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:prstGeom prst="rect"/>
+        <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -596,7 +596,7 @@
 </file>
 
 <file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>4</col>
@@ -604,21 +604,21 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5905500" cy="2032566"/>
+    <ext cx="5905500" cy="2008954"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:prstGeom prst="rect"/>
+        <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -629,7 +629,7 @@
 </file>
 
 <file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>10</col>
@@ -637,21 +637,21 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5905500" cy="4366955"/>
+    <ext cx="5905500" cy="4191502"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:prstGeom prst="rect"/>
+        <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -662,7 +662,7 @@
 </file>
 
 <file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>10</col>
@@ -670,21 +670,21 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5905500" cy="2764389"/>
+    <ext cx="5905500" cy="2711867"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:prstGeom prst="rect"/>
+        <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -4206,9 +4206,7 @@
       <c r="R4" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="S4" s="15" t="n">
-        <v>3099</v>
-      </c>
+      <c r="S4" s="15" t="n"/>
       <c r="T4" s="15" t="n">
         <v>76</v>
       </c>
@@ -4315,9 +4313,7 @@
       <c r="S5" s="15" t="n">
         <v>702</v>
       </c>
-      <c r="T5" s="15" t="n">
-        <v>1505</v>
-      </c>
+      <c r="T5" s="15" t="n"/>
       <c r="U5" s="15" t="n">
         <v>6058</v>
       </c>
@@ -4712,9 +4708,7 @@
       <c r="R8" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="S8" s="15" t="n">
-        <v>6361</v>
-      </c>
+      <c r="S8" s="15" t="n"/>
       <c r="T8" s="15" t="n">
         <v>162</v>
       </c>
@@ -4944,9 +4938,7 @@
       <c r="R10" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="S10" s="15" t="n">
-        <v>3702</v>
-      </c>
+      <c r="S10" s="15" t="n"/>
       <c r="T10" s="15" t="n">
         <v>228</v>
       </c>
@@ -5170,12 +5162,8 @@
       <c r="R12" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="S12" s="15" t="n">
-        <v>5144</v>
-      </c>
-      <c r="T12" s="15" t="n">
-        <v>1138</v>
-      </c>
+      <c r="S12" s="15" t="n"/>
+      <c r="T12" s="15" t="n"/>
       <c r="U12" s="15" t="n">
         <v>27673</v>
       </c>
@@ -5453,7 +5441,7 @@
         <v>0.01614</v>
       </c>
       <c r="AA14" s="15" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="AB14" s="15" t="n">
         <v>1</v>
@@ -5471,7 +5459,7 @@
         <v>35</v>
       </c>
       <c r="AG14" s="14" t="n">
-        <v>32.5</v>
+        <v>30</v>
       </c>
       <c r="AH14" s="14" t="n">
         <v>48</v>
@@ -5480,7 +5468,7 @@
         <v>54.5</v>
       </c>
       <c r="AJ14" s="14" t="n">
-        <v>56.75</v>
+        <v>54.25</v>
       </c>
       <c r="AK14" s="14" t="n">
         <v>73.5</v>
@@ -5492,7 +5480,7 @@
         <v>40</v>
       </c>
       <c r="AN14" s="14" t="n">
-        <v>31</v>
+        <v>30.5</v>
       </c>
       <c r="AO14" s="14" t="n">
         <v>13</v>
@@ -5694,9 +5682,7 @@
       <c r="R16" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="S16" s="15" t="n">
-        <v>1142</v>
-      </c>
+      <c r="S16" s="15" t="n"/>
       <c r="T16" s="15" t="n">
         <v>105</v>
       </c>
@@ -5830,9 +5816,7 @@
       <c r="R17" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="S17" s="15" t="n">
-        <v>1201</v>
-      </c>
+      <c r="S17" s="15" t="n"/>
       <c r="T17" s="15" t="n">
         <v>754</v>
       </c>
@@ -5854,12 +5838,18 @@
       <c r="Z17" s="16" t="n">
         <v>0.00134</v>
       </c>
-      <c r="AA17" s="15" t="n"/>
+      <c r="AA17" s="15" t="n">
+        <v>1</v>
+      </c>
       <c r="AB17" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC17" s="15" t="n"/>
-      <c r="AD17" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AC17" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD17" s="14" t="n">
+        <v>10</v>
+      </c>
       <c r="AE17" s="14" t="n"/>
       <c r="AF17" s="14" t="n"/>
       <c r="AG17" s="14" t="n"/>
@@ -5936,9 +5926,7 @@
       <c r="R18" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="S18" s="15" t="n">
-        <v>4984</v>
-      </c>
+      <c r="S18" s="15" t="n"/>
       <c r="T18" s="15" t="n">
         <v>137</v>
       </c>
@@ -6070,9 +6058,7 @@
       <c r="R19" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="S19" s="15" t="n">
-        <v>3205</v>
-      </c>
+      <c r="S19" s="15" t="n"/>
       <c r="T19" s="15" t="n">
         <v>391</v>
       </c>
@@ -6082,25 +6068,49 @@
       <c r="X19" s="15" t="n"/>
       <c r="Y19" s="14" t="n"/>
       <c r="Z19" s="16" t="n"/>
-      <c r="AA19" s="15" t="n"/>
+      <c r="AA19" s="15" t="n">
+        <v>11</v>
+      </c>
       <c r="AB19" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC19" s="15" t="n"/>
-      <c r="AD19" s="14" t="n"/>
-      <c r="AE19" s="14" t="n"/>
-      <c r="AF19" s="14" t="n"/>
-      <c r="AG19" s="14" t="n"/>
-      <c r="AH19" s="14" t="n"/>
-      <c r="AI19" s="14" t="n"/>
-      <c r="AJ19" s="14" t="n"/>
-      <c r="AK19" s="14" t="n"/>
-      <c r="AL19" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AC19" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD19" s="14" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="AE19" s="14" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="AF19" s="14" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="AG19" s="14" t="n">
+        <v>69.3</v>
+      </c>
+      <c r="AH19" s="14" t="n">
+        <v>73.3</v>
+      </c>
+      <c r="AI19" s="14" t="n">
+        <v>75.8</v>
+      </c>
+      <c r="AJ19" s="14" t="n">
+        <v>88.05</v>
+      </c>
+      <c r="AK19" s="14" t="n">
+        <v>95.8</v>
+      </c>
+      <c r="AL19" s="14" t="n">
+        <v>102.05</v>
+      </c>
       <c r="AM19" s="14" t="n"/>
       <c r="AN19" s="14" t="n"/>
       <c r="AO19" s="14" t="n"/>
       <c r="AP19" s="14" t="n"/>
-      <c r="AQ19" s="14" t="n"/>
+      <c r="AQ19" s="14" t="n">
+        <v>38.9</v>
+      </c>
       <c r="AR19" s="15" t="n">
         <v>362</v>
       </c>
@@ -6166,9 +6176,7 @@
       <c r="R20" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="S20" s="15" t="n">
-        <v>2556</v>
-      </c>
+      <c r="S20" s="15" t="n"/>
       <c r="T20" s="15" t="n">
         <v>221</v>
       </c>
@@ -6330,12 +6338,18 @@
       <c r="Z21" s="16" t="n">
         <v>0.00223</v>
       </c>
-      <c r="AA21" s="15" t="n"/>
+      <c r="AA21" s="15" t="n">
+        <v>2</v>
+      </c>
       <c r="AB21" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC21" s="15" t="n"/>
-      <c r="AD21" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AC21" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD21" s="14" t="n">
+        <v>20</v>
+      </c>
       <c r="AE21" s="14" t="n"/>
       <c r="AF21" s="14" t="n"/>
       <c r="AG21" s="14" t="n"/>
@@ -6542,9 +6556,7 @@
       <c r="R23" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="S23" s="15" t="n">
-        <v>1216</v>
-      </c>
+      <c r="S23" s="15" t="n"/>
       <c r="T23" s="15" t="n">
         <v>312</v>
       </c>
@@ -6754,9 +6766,7 @@
       <c r="R25" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="S25" s="15" t="n">
-        <v>7638</v>
-      </c>
+      <c r="S25" s="15" t="n"/>
       <c r="T25" s="15" t="n">
         <v>153</v>
       </c>
@@ -6772,25 +6782,49 @@
         <v>207.62</v>
       </c>
       <c r="Z25" s="16" t="n"/>
-      <c r="AA25" s="15" t="n"/>
+      <c r="AA25" s="15" t="n">
+        <v>75</v>
+      </c>
       <c r="AB25" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC25" s="15" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AC25" s="15" t="n">
+        <v>0</v>
+      </c>
       <c r="AD25" s="14" t="n"/>
-      <c r="AE25" s="14" t="n"/>
-      <c r="AF25" s="14" t="n"/>
-      <c r="AG25" s="14" t="n"/>
-      <c r="AH25" s="14" t="n"/>
-      <c r="AI25" s="14" t="n"/>
+      <c r="AE25" s="14" t="n">
+        <v>25</v>
+      </c>
+      <c r="AF25" s="14" t="n">
+        <v>36</v>
+      </c>
+      <c r="AG25" s="14" t="n">
+        <v>41</v>
+      </c>
+      <c r="AH25" s="14" t="n">
+        <v>61</v>
+      </c>
+      <c r="AI25" s="14" t="n">
+        <v>75.75</v>
+      </c>
       <c r="AJ25" s="14" t="n"/>
       <c r="AK25" s="14" t="n"/>
       <c r="AL25" s="14" t="n"/>
-      <c r="AM25" s="14" t="n"/>
-      <c r="AN25" s="14" t="n"/>
-      <c r="AO25" s="14" t="n"/>
-      <c r="AP25" s="14" t="n"/>
-      <c r="AQ25" s="14" t="n"/>
+      <c r="AM25" s="14" t="n">
+        <v>49</v>
+      </c>
+      <c r="AN25" s="14" t="n">
+        <v>22</v>
+      </c>
+      <c r="AO25" s="14" t="n">
+        <v>23</v>
+      </c>
+      <c r="AP25" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="AQ25" s="14" t="n">
+        <v>32</v>
+      </c>
       <c r="AR25" s="15" t="n">
         <v>1357</v>
       </c>
@@ -6859,9 +6893,7 @@
       <c r="S26" s="15" t="n">
         <v>351</v>
       </c>
-      <c r="T26" s="15" t="n">
-        <v>1796</v>
-      </c>
+      <c r="T26" s="15" t="n"/>
       <c r="U26" s="15" t="n">
         <v>6682</v>
       </c>
@@ -6881,7 +6913,7 @@
         <v>0.00353</v>
       </c>
       <c r="AA26" s="15" t="n">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="AB26" s="15" t="n">
         <v>1</v>
@@ -6896,28 +6928,28 @@
         <v>11</v>
       </c>
       <c r="AF26" s="14" t="n">
-        <v>45</v>
+        <v>39.5</v>
       </c>
       <c r="AG26" s="14" t="n">
-        <v>46</v>
+        <v>43.25</v>
       </c>
       <c r="AH26" s="14" t="n">
-        <v>56</v>
+        <v>50.5</v>
       </c>
       <c r="AI26" s="14" t="n">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="AJ26" s="14" t="n">
-        <v>52.25</v>
+        <v>49.5</v>
       </c>
       <c r="AK26" s="14" t="n">
-        <v>68.5</v>
+        <v>63</v>
       </c>
       <c r="AL26" s="14" t="n">
-        <v>96.75</v>
+        <v>83.75</v>
       </c>
       <c r="AM26" s="14" t="n">
-        <v>52.5</v>
+        <v>42</v>
       </c>
       <c r="AN26" s="14" t="n">
         <v>28.5</v>
@@ -7021,7 +7053,7 @@
         <v>0.00153</v>
       </c>
       <c r="AA27" s="15" t="n">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="AB27" s="15" t="n">
         <v>1</v>
@@ -7043,7 +7075,7 @@
         <v>60</v>
       </c>
       <c r="AI27" s="14" t="n">
-        <v>76</v>
+        <v>77.5</v>
       </c>
       <c r="AJ27" s="14" t="n"/>
       <c r="AK27" s="14" t="n"/>
@@ -7055,7 +7087,7 @@
         <v>39</v>
       </c>
       <c r="AO27" s="14" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="AP27" s="14" t="n">
         <v>8</v>
@@ -7128,9 +7160,7 @@
       <c r="R28" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="S28" s="15" t="n">
-        <v>10228</v>
-      </c>
+      <c r="S28" s="15" t="n"/>
       <c r="T28" s="15" t="n">
         <v>684</v>
       </c>
@@ -7359,9 +7389,7 @@
       <c r="S30" s="15" t="n">
         <v>577</v>
       </c>
-      <c r="T30" s="15" t="n">
-        <v>1006</v>
-      </c>
+      <c r="T30" s="15" t="n"/>
       <c r="U30" s="15" t="n">
         <v>41545</v>
       </c>
@@ -7381,7 +7409,7 @@
         <v>0.00048</v>
       </c>
       <c r="AA30" s="15" t="n">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="AB30" s="15" t="n">
         <v>1</v>
@@ -7391,16 +7419,16 @@
       </c>
       <c r="AD30" s="14" t="n"/>
       <c r="AE30" s="14" t="n">
-        <v>28.4</v>
+        <v>26.9</v>
       </c>
       <c r="AF30" s="14" t="n">
         <v>43.4</v>
       </c>
       <c r="AG30" s="14" t="n">
-        <v>55.57</v>
+        <v>54.15</v>
       </c>
       <c r="AH30" s="14" t="n">
-        <v>71.8</v>
+        <v>70.3</v>
       </c>
       <c r="AI30" s="14" t="n">
         <v>83.55</v>
@@ -7421,7 +7449,7 @@
         <v>9</v>
       </c>
       <c r="AQ30" s="14" t="n">
-        <v>37.9</v>
+        <v>37.4</v>
       </c>
       <c r="AR30" s="15" t="n">
         <v>225</v>
@@ -7513,7 +7541,7 @@
         <v>0.00419</v>
       </c>
       <c r="AA31" s="15" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AB31" s="15" t="n">
         <v>1</v>
@@ -7529,7 +7557,7 @@
         <v>32</v>
       </c>
       <c r="AG31" s="14" t="n">
-        <v>47.75</v>
+        <v>47.5</v>
       </c>
       <c r="AH31" s="14" t="n">
         <v>60</v>
@@ -7544,7 +7572,7 @@
         <v>28</v>
       </c>
       <c r="AN31" s="14" t="n">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="AO31" s="14" t="n">
         <v>22</v>
@@ -7618,9 +7646,7 @@
       <c r="R32" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="S32" s="15" t="n">
-        <v>7180</v>
-      </c>
+      <c r="S32" s="15" t="n"/>
       <c r="T32" s="15" t="n">
         <v>424</v>
       </c>
@@ -7750,12 +7776,8 @@
       <c r="R33" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="S33" s="15" t="n">
-        <v>16823</v>
-      </c>
-      <c r="T33" s="15" t="n">
-        <v>1993</v>
-      </c>
+      <c r="S33" s="15" t="n"/>
+      <c r="T33" s="15" t="n"/>
       <c r="U33" s="15" t="n">
         <v>2732</v>
       </c>
@@ -8009,9 +8031,7 @@
       <c r="S35" s="15" t="n">
         <v>628</v>
       </c>
-      <c r="T35" s="15" t="n">
-        <v>1205</v>
-      </c>
+      <c r="T35" s="15" t="n"/>
       <c r="U35" s="15" t="n">
         <v>110000</v>
       </c>
@@ -8030,22 +8050,48 @@
       <c r="Z35" s="16" t="n">
         <v>0.00117</v>
       </c>
-      <c r="AA35" s="15" t="n"/>
+      <c r="AA35" s="15" t="n">
+        <v>27</v>
+      </c>
       <c r="AB35" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC35" s="15" t="n"/>
-      <c r="AD35" s="14" t="n"/>
-      <c r="AE35" s="14" t="n"/>
-      <c r="AF35" s="14" t="n"/>
-      <c r="AG35" s="14" t="n"/>
-      <c r="AH35" s="14" t="n"/>
-      <c r="AI35" s="14" t="n"/>
-      <c r="AJ35" s="14" t="n"/>
-      <c r="AK35" s="14" t="n"/>
-      <c r="AL35" s="14" t="n"/>
-      <c r="AM35" s="14" t="n"/>
-      <c r="AN35" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AC35" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD35" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="AE35" s="14" t="n">
+        <v>32.4</v>
+      </c>
+      <c r="AF35" s="14" t="n">
+        <v>37.3</v>
+      </c>
+      <c r="AG35" s="14" t="n">
+        <v>58.35</v>
+      </c>
+      <c r="AH35" s="14" t="n">
+        <v>69.7</v>
+      </c>
+      <c r="AI35" s="14" t="n">
+        <v>87.8</v>
+      </c>
+      <c r="AJ35" s="14" t="n">
+        <v>78.34999999999999</v>
+      </c>
+      <c r="AK35" s="14" t="n">
+        <v>89.7</v>
+      </c>
+      <c r="AL35" s="14" t="n">
+        <v>107.8</v>
+      </c>
+      <c r="AM35" s="14" t="n">
+        <v>50.3</v>
+      </c>
+      <c r="AN35" s="14" t="n">
+        <v>26.7</v>
+      </c>
       <c r="AO35" s="14" t="n"/>
       <c r="AP35" s="14" t="n"/>
       <c r="AQ35" s="14" t="n"/>
@@ -8497,9 +8543,7 @@
       <c r="S39" s="15" t="n">
         <v>820</v>
       </c>
-      <c r="T39" s="15" t="n">
-        <v>1083</v>
-      </c>
+      <c r="T39" s="15" t="n"/>
       <c r="U39" s="15" t="n">
         <v>8510</v>
       </c>
@@ -8605,9 +8649,7 @@
       <c r="S40" s="15" t="n">
         <v>566</v>
       </c>
-      <c r="T40" s="15" t="n">
-        <v>1744</v>
-      </c>
+      <c r="T40" s="15" t="n"/>
       <c r="U40" s="15" t="n">
         <v>23415</v>
       </c>
@@ -8710,9 +8752,7 @@
       <c r="R41" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="S41" s="15" t="n">
-        <v>4310</v>
-      </c>
+      <c r="S41" s="15" t="n"/>
       <c r="T41" s="15" t="n">
         <v>251</v>
       </c>
@@ -8735,7 +8775,7 @@
         <v>0.0064</v>
       </c>
       <c r="AA41" s="15" t="n">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="AB41" s="15" t="n">
         <v>1</v>
@@ -8745,19 +8785,19 @@
       </c>
       <c r="AD41" s="14" t="n"/>
       <c r="AE41" s="14" t="n">
-        <v>10.5</v>
+        <v>9</v>
       </c>
       <c r="AF41" s="14" t="n">
         <v>29</v>
       </c>
       <c r="AG41" s="14" t="n">
-        <v>18.18</v>
+        <v>17.9</v>
       </c>
       <c r="AH41" s="14" t="n">
-        <v>39.5</v>
+        <v>38</v>
       </c>
       <c r="AI41" s="14" t="n">
-        <v>53.5</v>
+        <v>52.72</v>
       </c>
       <c r="AJ41" s="14" t="n"/>
       <c r="AK41" s="14" t="n"/>
@@ -8772,7 +8812,7 @@
         <v>13</v>
       </c>
       <c r="AP41" s="14" t="n">
-        <v>11</v>
+        <v>6.9</v>
       </c>
       <c r="AQ41" s="14" t="n"/>
       <c r="AR41" s="15" t="n">
@@ -8968,9 +9008,7 @@
       <c r="R43" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="S43" s="15" t="n">
-        <v>1527</v>
-      </c>
+      <c r="S43" s="15" t="n"/>
       <c r="T43" s="15" t="n">
         <v>305</v>
       </c>
@@ -8989,7 +9027,7 @@
       </c>
       <c r="Z43" s="16" t="n"/>
       <c r="AA43" s="15" t="n">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="AB43" s="15" t="n">
         <v>1</v>
@@ -9009,7 +9047,7 @@
       <c r="AK43" s="14" t="n"/>
       <c r="AL43" s="14" t="n"/>
       <c r="AM43" s="14" t="n">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="AN43" s="14" t="n">
         <v>35</v>
@@ -9085,9 +9123,7 @@
       <c r="S44" s="15" t="n">
         <v>364</v>
       </c>
-      <c r="T44" s="15" t="n">
-        <v>1486</v>
-      </c>
+      <c r="T44" s="15" t="n"/>
       <c r="U44" s="15" t="n">
         <v>34668</v>
       </c>
@@ -9211,7 +9247,7 @@
         <v>0.00343</v>
       </c>
       <c r="AA45" s="15" t="n">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="AB45" s="15" t="n">
         <v>1</v>
@@ -9335,7 +9371,7 @@
         <v>0.00173</v>
       </c>
       <c r="AA46" s="15" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="AB46" s="15" t="n">
         <v>1</v>
@@ -9351,13 +9387,13 @@
         <v>12</v>
       </c>
       <c r="AG46" s="14" t="n">
-        <v>22</v>
+        <v>21.75</v>
       </c>
       <c r="AH46" s="14" t="n">
         <v>24</v>
       </c>
       <c r="AI46" s="14" t="n">
-        <v>34</v>
+        <v>28.5</v>
       </c>
       <c r="AJ46" s="14" t="n"/>
       <c r="AK46" s="14" t="n"/>
@@ -9435,9 +9471,7 @@
         <v>0</v>
       </c>
       <c r="S47" s="15" t="n"/>
-      <c r="T47" s="15" t="n">
-        <v>1175</v>
-      </c>
+      <c r="T47" s="15" t="n"/>
       <c r="U47" s="15" t="n">
         <v>18698</v>
       </c>
@@ -9457,7 +9491,7 @@
         <v>0.00693</v>
       </c>
       <c r="AA47" s="15" t="n">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="AB47" s="15" t="n">
         <v>1</v>
@@ -9467,31 +9501,31 @@
       </c>
       <c r="AD47" s="14" t="n"/>
       <c r="AE47" s="14" t="n">
-        <v>17.5</v>
+        <v>16</v>
       </c>
       <c r="AF47" s="14" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="AG47" s="14" t="n">
-        <v>43</v>
+        <v>41.75</v>
       </c>
       <c r="AH47" s="14" t="n">
-        <v>47.5</v>
+        <v>44</v>
       </c>
       <c r="AI47" s="14" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="AJ47" s="14" t="n"/>
       <c r="AK47" s="14" t="n"/>
       <c r="AL47" s="14" t="n"/>
       <c r="AM47" s="14" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="AN47" s="14" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="AO47" s="14" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="AP47" s="14" t="n">
         <v>8</v>
@@ -9563,9 +9597,7 @@
         <v>0</v>
       </c>
       <c r="S48" s="15" t="n"/>
-      <c r="T48" s="15" t="n">
-        <v>1152</v>
-      </c>
+      <c r="T48" s="15" t="n"/>
       <c r="U48" s="15" t="n">
         <v>25555</v>
       </c>
@@ -9584,12 +9616,18 @@
       <c r="Z48" s="16" t="n">
         <v>0.01197</v>
       </c>
-      <c r="AA48" s="15" t="n"/>
+      <c r="AA48" s="15" t="n">
+        <v>2</v>
+      </c>
       <c r="AB48" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC48" s="15" t="n"/>
-      <c r="AD48" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AC48" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD48" s="14" t="n">
+        <v>12.5</v>
+      </c>
       <c r="AE48" s="14" t="n"/>
       <c r="AF48" s="14" t="n"/>
       <c r="AG48" s="14" t="n"/>
@@ -10003,7 +10041,7 @@
         <v>0.03043</v>
       </c>
       <c r="AA52" s="15" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AB52" s="15" t="n">
         <v>1</v>
@@ -10026,7 +10064,7 @@
         <v>36</v>
       </c>
       <c r="AN52" s="14" t="n">
-        <v>54</v>
+        <v>44.5</v>
       </c>
       <c r="AO52" s="14" t="n"/>
       <c r="AP52" s="14" t="n"/>
@@ -10113,7 +10151,7 @@
       <c r="Y53" s="14" t="n"/>
       <c r="Z53" s="16" t="n"/>
       <c r="AA53" s="15" t="n">
-        <v>100</v>
+        <v>72</v>
       </c>
       <c r="AB53" s="15" t="n">
         <v>1</v>
@@ -10129,13 +10167,13 @@
         <v>25.9</v>
       </c>
       <c r="AG53" s="14" t="n">
-        <v>28.4</v>
+        <v>30.4</v>
       </c>
       <c r="AH53" s="14" t="n">
         <v>32.7</v>
       </c>
       <c r="AI53" s="14" t="n">
-        <v>37.6</v>
+        <v>43.6</v>
       </c>
       <c r="AJ53" s="14" t="n"/>
       <c r="AK53" s="14" t="n"/>
@@ -10215,9 +10253,7 @@
         <v>0</v>
       </c>
       <c r="S54" s="15" t="n"/>
-      <c r="T54" s="15" t="n">
-        <v>1681</v>
-      </c>
+      <c r="T54" s="15" t="n"/>
       <c r="U54" s="15" t="n">
         <v>87929</v>
       </c>
@@ -10237,7 +10273,7 @@
         <v>0.0023</v>
       </c>
       <c r="AA54" s="15" t="n">
-        <v>137</v>
+        <v>112</v>
       </c>
       <c r="AB54" s="15" t="n">
         <v>1</v>
@@ -10250,16 +10286,16 @@
         <v>17.9</v>
       </c>
       <c r="AF54" s="14" t="n">
-        <v>30.9</v>
+        <v>31.9</v>
       </c>
       <c r="AG54" s="14" t="n">
-        <v>34.9</v>
+        <v>35.55</v>
       </c>
       <c r="AH54" s="14" t="n">
-        <v>48.8</v>
+        <v>49.8</v>
       </c>
       <c r="AI54" s="14" t="n">
-        <v>67.67</v>
+        <v>71.42</v>
       </c>
       <c r="AJ54" s="14" t="n"/>
       <c r="AK54" s="14" t="n"/>
@@ -10277,7 +10313,7 @@
         <v>6.75</v>
       </c>
       <c r="AQ54" s="14" t="n">
-        <v>20.9</v>
+        <v>21.4</v>
       </c>
       <c r="AR54" s="15" t="n"/>
     </row>
@@ -10342,9 +10378,7 @@
       <c r="R55" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="S55" s="15" t="n">
-        <v>1300</v>
-      </c>
+      <c r="S55" s="15" t="n"/>
       <c r="T55" s="15" t="n">
         <v>591</v>
       </c>
@@ -10367,7 +10401,7 @@
         <v>0.00084</v>
       </c>
       <c r="AA55" s="15" t="n">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="AB55" s="15" t="n">
         <v>1</v>
@@ -10383,13 +10417,13 @@
         <v>40</v>
       </c>
       <c r="AG55" s="14" t="n">
-        <v>52.75</v>
+        <v>55</v>
       </c>
       <c r="AH55" s="14" t="n">
         <v>65</v>
       </c>
       <c r="AI55" s="14" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="AJ55" s="14" t="n"/>
       <c r="AK55" s="14" t="n"/>
@@ -10401,7 +10435,7 @@
         <v>28</v>
       </c>
       <c r="AO55" s="14" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="AP55" s="14" t="n">
         <v>8</v>
@@ -10472,9 +10506,7 @@
       <c r="R56" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="S56" s="19" t="n">
-        <v>15504</v>
-      </c>
+      <c r="S56" s="19" t="n"/>
       <c r="T56" s="19" t="n">
         <v>583</v>
       </c>

</xml_diff>

<commit_message>
B1: couvert de 10 casas a partir de prints do Instagram, com caps. 3, 5, 6 e 9 e Notion atualizados
O autor achou no Instagram a taxa de entrada de TabuClub, Café Geek,
Tubaleria, Place Games, Encounter, Covil, Luderia Carioca, Bardo Mago,
Toca do Rato e Nala Land. Com elas, 21 dos 53 concorrentes têm a taxa
conhecida (mediana de R$ 20,00; R$ 25,00 no fim de semana), contra 8 no
texto anterior. O crepe "Lúdico" da Ludoteca BGC saiu da categoria de
couvert. A conclusão do preço não muda: a São Jogue fica acima da mediana.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/Dados agregados/B1_dados_agregados_completo.xlsx
+++ b/dados/Dados agregados/B1_dados_agregados_completo.xlsx
@@ -4603,11 +4603,9 @@
         <v>1</v>
       </c>
       <c r="AC7" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD7" s="14" t="n">
-        <v>30</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AD7" s="14" t="n"/>
       <c r="AE7" s="14" t="n">
         <v>9</v>
       </c>
@@ -4615,7 +4613,7 @@
         <v>31</v>
       </c>
       <c r="AG7" s="14" t="n">
-        <v>34.5</v>
+        <v>34.75</v>
       </c>
       <c r="AH7" s="14" t="n">
         <v>40</v>
@@ -4623,15 +4621,9 @@
       <c r="AI7" s="14" t="n">
         <v>46.75</v>
       </c>
-      <c r="AJ7" s="14" t="n">
-        <v>64.5</v>
-      </c>
-      <c r="AK7" s="14" t="n">
-        <v>70</v>
-      </c>
-      <c r="AL7" s="14" t="n">
-        <v>76.75</v>
-      </c>
+      <c r="AJ7" s="14" t="n"/>
+      <c r="AK7" s="14" t="n"/>
+      <c r="AL7" s="14" t="n"/>
       <c r="AM7" s="14" t="n"/>
       <c r="AN7" s="14" t="n"/>
       <c r="AO7" s="14" t="n">
@@ -5183,15 +5175,17 @@
         <v>0.00249</v>
       </c>
       <c r="AA12" s="15" t="n">
+        <v>28</v>
+      </c>
+      <c r="AB12" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC12" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD12" s="14" t="n">
         <v>25</v>
       </c>
-      <c r="AB12" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC12" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD12" s="14" t="n"/>
       <c r="AE12" s="14" t="n">
         <v>12</v>
       </c>
@@ -5207,9 +5201,15 @@
       <c r="AI12" s="14" t="n">
         <v>37.5</v>
       </c>
-      <c r="AJ12" s="14" t="n"/>
-      <c r="AK12" s="14" t="n"/>
-      <c r="AL12" s="14" t="n"/>
+      <c r="AJ12" s="14" t="n">
+        <v>52</v>
+      </c>
+      <c r="AK12" s="14" t="n">
+        <v>59</v>
+      </c>
+      <c r="AL12" s="14" t="n">
+        <v>62.5</v>
+      </c>
       <c r="AM12" s="14" t="n">
         <v>34</v>
       </c>
@@ -5577,15 +5577,17 @@
       </c>
       <c r="Z15" s="16" t="n"/>
       <c r="AA15" s="15" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="AB15" s="15" t="n">
         <v>1</v>
       </c>
       <c r="AC15" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD15" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AD15" s="14" t="n">
+        <v>20</v>
+      </c>
       <c r="AE15" s="14" t="n">
         <v>20</v>
       </c>
@@ -5601,9 +5603,15 @@
       <c r="AI15" s="14" t="n">
         <v>71.5</v>
       </c>
-      <c r="AJ15" s="14" t="n"/>
-      <c r="AK15" s="14" t="n"/>
-      <c r="AL15" s="14" t="n"/>
+      <c r="AJ15" s="14" t="n">
+        <v>58</v>
+      </c>
+      <c r="AK15" s="14" t="n">
+        <v>74</v>
+      </c>
+      <c r="AL15" s="14" t="n">
+        <v>94</v>
+      </c>
       <c r="AM15" s="14" t="n">
         <v>42</v>
       </c>
@@ -6451,15 +6459,17 @@
         <v>0.01027</v>
       </c>
       <c r="AA22" s="15" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="AB22" s="15" t="n">
         <v>1</v>
       </c>
       <c r="AC22" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD22" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AD22" s="14" t="n">
+        <v>20</v>
+      </c>
       <c r="AE22" s="14" t="n">
         <v>12</v>
       </c>
@@ -6475,9 +6485,15 @@
       <c r="AI22" s="14" t="n">
         <v>54.5</v>
       </c>
-      <c r="AJ22" s="14" t="n"/>
-      <c r="AK22" s="14" t="n"/>
-      <c r="AL22" s="14" t="n"/>
+      <c r="AJ22" s="14" t="n">
+        <v>55</v>
+      </c>
+      <c r="AK22" s="14" t="n">
+        <v>64</v>
+      </c>
+      <c r="AL22" s="14" t="n">
+        <v>74.5</v>
+      </c>
       <c r="AM22" s="14" t="n">
         <v>38</v>
       </c>
@@ -6783,15 +6799,17 @@
       </c>
       <c r="Z25" s="16" t="n"/>
       <c r="AA25" s="15" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="AB25" s="15" t="n">
         <v>1</v>
       </c>
       <c r="AC25" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD25" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AD25" s="14" t="n">
+        <v>22.5</v>
+      </c>
       <c r="AE25" s="14" t="n">
         <v>25</v>
       </c>
@@ -6807,9 +6825,15 @@
       <c r="AI25" s="14" t="n">
         <v>75.75</v>
       </c>
-      <c r="AJ25" s="14" t="n"/>
-      <c r="AK25" s="14" t="n"/>
-      <c r="AL25" s="14" t="n"/>
+      <c r="AJ25" s="14" t="n">
+        <v>62.25</v>
+      </c>
+      <c r="AK25" s="14" t="n">
+        <v>83.5</v>
+      </c>
+      <c r="AL25" s="14" t="n">
+        <v>99.5</v>
+      </c>
       <c r="AM25" s="14" t="n">
         <v>49</v>
       </c>
@@ -7669,15 +7693,17 @@
         <v>0.03412</v>
       </c>
       <c r="AA32" s="15" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="AB32" s="15" t="n">
         <v>1</v>
       </c>
       <c r="AC32" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD32" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AD32" s="14" t="n">
+        <v>17.5</v>
+      </c>
       <c r="AE32" s="14" t="n">
         <v>18</v>
       </c>
@@ -7693,9 +7719,15 @@
       <c r="AI32" s="14" t="n">
         <v>60</v>
       </c>
-      <c r="AJ32" s="14" t="n"/>
-      <c r="AK32" s="14" t="n"/>
-      <c r="AL32" s="14" t="n"/>
+      <c r="AJ32" s="14" t="n">
+        <v>59.25</v>
+      </c>
+      <c r="AK32" s="14" t="n">
+        <v>69.5</v>
+      </c>
+      <c r="AL32" s="14" t="n">
+        <v>78.75</v>
+      </c>
       <c r="AM32" s="14" t="n">
         <v>29</v>
       </c>
@@ -7929,15 +7961,17 @@
         <v>0.00322</v>
       </c>
       <c r="AA34" s="15" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="AB34" s="15" t="n">
         <v>1</v>
       </c>
       <c r="AC34" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD34" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AD34" s="14" t="n">
+        <v>40</v>
+      </c>
       <c r="AE34" s="14" t="n">
         <v>27.9</v>
       </c>
@@ -7953,9 +7987,15 @@
       <c r="AI34" s="14" t="n">
         <v>76.8</v>
       </c>
-      <c r="AJ34" s="14" t="n"/>
-      <c r="AK34" s="14" t="n"/>
-      <c r="AL34" s="14" t="n"/>
+      <c r="AJ34" s="14" t="n">
+        <v>101.55</v>
+      </c>
+      <c r="AK34" s="14" t="n">
+        <v>107.8</v>
+      </c>
+      <c r="AL34" s="14" t="n">
+        <v>118.05</v>
+      </c>
       <c r="AM34" s="14" t="n">
         <v>38</v>
       </c>
@@ -8775,15 +8815,17 @@
         <v>0.0064</v>
       </c>
       <c r="AA41" s="15" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="AB41" s="15" t="n">
         <v>1</v>
       </c>
       <c r="AC41" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD41" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AD41" s="14" t="n">
+        <v>12.5</v>
+      </c>
       <c r="AE41" s="14" t="n">
         <v>9</v>
       </c>
@@ -8799,9 +8841,15 @@
       <c r="AI41" s="14" t="n">
         <v>52.72</v>
       </c>
-      <c r="AJ41" s="14" t="n"/>
-      <c r="AK41" s="14" t="n"/>
-      <c r="AL41" s="14" t="n"/>
+      <c r="AJ41" s="14" t="n">
+        <v>24.15</v>
+      </c>
+      <c r="AK41" s="14" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="AL41" s="14" t="n">
+        <v>71.47</v>
+      </c>
       <c r="AM41" s="14" t="n">
         <v>38.9</v>
       </c>
@@ -9027,15 +9075,17 @@
       </c>
       <c r="Z43" s="16" t="n"/>
       <c r="AA43" s="15" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AB43" s="15" t="n">
         <v>1</v>
       </c>
       <c r="AC43" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD43" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AD43" s="14" t="n">
+        <v>28</v>
+      </c>
       <c r="AE43" s="14" t="n"/>
       <c r="AF43" s="14" t="n">
         <v>38</v>
@@ -9247,15 +9297,17 @@
         <v>0.00343</v>
       </c>
       <c r="AA45" s="15" t="n">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="AB45" s="15" t="n">
         <v>1</v>
       </c>
       <c r="AC45" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD45" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AD45" s="14" t="n">
+        <v>10</v>
+      </c>
       <c r="AE45" s="14" t="n">
         <v>12.5</v>
       </c>
@@ -9271,9 +9323,15 @@
       <c r="AI45" s="14" t="n">
         <v>30.25</v>
       </c>
-      <c r="AJ45" s="14" t="n"/>
-      <c r="AK45" s="14" t="n"/>
-      <c r="AL45" s="14" t="n"/>
+      <c r="AJ45" s="14" t="n">
+        <v>22.75</v>
+      </c>
+      <c r="AK45" s="14" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="AL45" s="14" t="n">
+        <v>42.25</v>
+      </c>
       <c r="AM45" s="14" t="n"/>
       <c r="AN45" s="14" t="n">
         <v>18</v>
@@ -10523,15 +10581,17 @@
       </c>
       <c r="Z56" s="20" t="n"/>
       <c r="AA56" s="19" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AB56" s="19" t="n">
         <v>1</v>
       </c>
       <c r="AC56" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD56" s="18" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AD56" s="18" t="n">
+        <v>5</v>
+      </c>
       <c r="AE56" s="18" t="n">
         <v>7.5</v>
       </c>
@@ -10547,9 +10607,15 @@
       <c r="AI56" s="18" t="n">
         <v>81.5</v>
       </c>
-      <c r="AJ56" s="18" t="n"/>
-      <c r="AK56" s="18" t="n"/>
-      <c r="AL56" s="18" t="n"/>
+      <c r="AJ56" s="18" t="n">
+        <v>69.67</v>
+      </c>
+      <c r="AK56" s="18" t="n">
+        <v>76.95</v>
+      </c>
+      <c r="AL56" s="18" t="n">
+        <v>86.5</v>
+      </c>
       <c r="AM56" s="18" t="n"/>
       <c r="AN56" s="18" t="n"/>
       <c r="AO56" s="18" t="n"/>

</xml_diff>

<commit_message>
B1: couvert de BoardZ e LudoCafé, com caps. 5, 6 e 9 e Notion atualizados
Prints enviados pelo autor: Day Pass da BoardZ (site) e cartaz do couvert lúdico
do LudoCafé, que substitui o valor de imprensa de 2024. Game of Boards confirmado.
Agora 22 dos 53 concorrentes cobram; medianas da Tabela 6.1 sem mudança.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/Dados agregados/B1_dados_agregados_completo.xlsx
+++ b/dados/Dados agregados/B1_dados_agregados_completo.xlsx
@@ -571,7 +571,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5905500" cy="3183595"/>
+    <ext cx="5905500" cy="3176182"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -6077,7 +6077,7 @@
       <c r="Y19" s="14" t="n"/>
       <c r="Z19" s="16" t="n"/>
       <c r="AA19" s="15" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="AB19" s="15" t="n">
         <v>1</v>
@@ -6104,13 +6104,13 @@
         <v>75.8</v>
       </c>
       <c r="AJ19" s="14" t="n">
-        <v>88.05</v>
+        <v>86.8</v>
       </c>
       <c r="AK19" s="14" t="n">
         <v>95.8</v>
       </c>
       <c r="AL19" s="14" t="n">
-        <v>102.05</v>
+        <v>103.3</v>
       </c>
       <c r="AM19" s="14" t="n"/>
       <c r="AN19" s="14" t="n"/>
@@ -9549,15 +9549,17 @@
         <v>0.00693</v>
       </c>
       <c r="AA47" s="15" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="AB47" s="15" t="n">
         <v>1</v>
       </c>
       <c r="AC47" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD47" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AD47" s="14" t="n">
+        <v>12.5</v>
+      </c>
       <c r="AE47" s="14" t="n">
         <v>16</v>
       </c>
@@ -9573,9 +9575,15 @@
       <c r="AI47" s="14" t="n">
         <v>57</v>
       </c>
-      <c r="AJ47" s="14" t="n"/>
-      <c r="AK47" s="14" t="n"/>
-      <c r="AL47" s="14" t="n"/>
+      <c r="AJ47" s="14" t="n">
+        <v>53</v>
+      </c>
+      <c r="AK47" s="14" t="n">
+        <v>56.5</v>
+      </c>
+      <c r="AL47" s="14" t="n">
+        <v>70.75</v>
+      </c>
       <c r="AM47" s="14" t="n">
         <v>28</v>
       </c>

</xml_diff>